<commit_message>
Lock Roman Gold Belt and Venus as 2025 art sales.
Belt is a Fortuna-to-L5 dealer sale (cost $45,000, L5 $50,000, net $5,000).
Venus is a joint purchase remitted at EPGC proceeds $26,000 (net $6,000).
EPGC July Art Sales is $76,000; Income I8 is $34,055.06. Remaining EOEB/L5 stay unallocated.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
+++ b/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="169" formatCode="_([$CAD]\ * #,##0.00_);_([$CAD]\ * \(#,##0.00\);_([$CAD]\ * &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -218,6 +218,11 @@
       <name val="Century Gothic"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="32">
@@ -696,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="239">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1195,6 +1200,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="36" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1694,8 +1708,8 @@
       <c r="H8" s="138" t="n">
         <v>20000</v>
       </c>
-      <c r="I8" s="139" t="n">
-        <v>23055.06</v>
+      <c r="I8" s="183" t="n">
+        <v>34055.06</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="137">
@@ -1769,9 +1783,9 @@
       <c r="B11" s="88" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1" s="137">
-      <c r="A12" s="191" t="inlineStr">
-        <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $23,055.06 = MATCHED Mercury deals only (Berk lots $30,000 − $22,944.94 Cost) + seals $1,000 + mosaics $15,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). Erdal/Aysel/EOEB/L5 ASK. Not tax advice.</t>
+      <c r="A12" s="182" t="inlineStr">
+        <is>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $34,055.06 = prior MATCHED nets $23,055.06 (Berk lots + seals $1,000 + mosaics $15,000) + Belt net $5,000 + Venus EPGC-share net $6,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 / other L5 $37,396.32 / other Erdal IN $31,000 / Aysel $50,000 / Fortuna Aug $20,000 still ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -8645,7 +8659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="137" min="1" max="1"/>
@@ -8870,29 +8884,29 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="224" t="inlineStr">
+      <c r="A11" s="226" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="B11" s="224" t="inlineStr">
+      <c r="B11" s="226" t="inlineStr">
         <is>
           <t>Art Sales net I8</t>
         </is>
       </c>
-      <c r="C11" s="224" t="inlineStr">
-        <is>
-          <t>23,055.06</t>
-        </is>
-      </c>
-      <c r="D11" s="224" t="inlineStr">
-        <is>
-          <t>MATCHED Mercury deals with Cost only (Berk lots + seals + mosaics). Sale 6428 and Aquinas books wait on Cost.</t>
+      <c r="C11" s="226" t="inlineStr">
+        <is>
+          <t>34,055.06</t>
+        </is>
+      </c>
+      <c r="D11" s="226" t="inlineStr">
+        <is>
+          <t>Prior MATCHED $23,055.06 + Belt net $5,000 + Venus EPGC-share net $6,000. Sale 6428 and Aquinas wait on Cost.</t>
         </is>
       </c>
       <c r="E11" s="226" t="inlineStr">
         <is>
-          <t>LOCKED</t>
+          <t>LOCKED green</t>
         </is>
       </c>
     </row>
@@ -9221,24 +9235,24 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="224" t="inlineStr">
+      <c r="A24" s="226" t="inlineStr">
         <is>
           <t>EPGC LLC</t>
         </is>
       </c>
-      <c r="B24" s="224" t="inlineStr">
+      <c r="B24" s="226" t="inlineStr">
         <is>
           <t>Art Sales</t>
         </is>
       </c>
-      <c r="C24" s="224" t="inlineStr">
-        <is>
-          <t>14,000 Jan + 136,000 Feb = 150,000</t>
-        </is>
-      </c>
-      <c r="D24" s="224" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED (Berk + mosaics + Aquinas cash). Do not dump EOEB/L5 remainder.</t>
+      <c r="C24" s="226" t="inlineStr">
+        <is>
+          <t>14,000 Jan + 136,000 Feb + 76,000 July = 226,000</t>
+        </is>
+      </c>
+      <c r="D24" s="226" t="inlineStr">
+        <is>
+          <t>Gross sale cash. July = Belt L5 $50,000 + Venus remittance $26,000. Do not dump EOEB $130,270 or other L5 $37,396.32.</t>
         </is>
       </c>
       <c r="E24" s="226" t="inlineStr">
@@ -9309,17 +9323,17 @@
       </c>
       <c r="B27" s="224" t="inlineStr">
         <is>
-          <t>Seals / lots / mosaics</t>
+          <t>Seals / lots / mosaics / Belt / Venus</t>
         </is>
       </c>
       <c r="C27" s="224" t="inlineStr">
         <is>
-          <t>see rows 70–74</t>
+          <t>rows 70–79</t>
         </is>
       </c>
       <c r="D27" s="224" t="inlineStr">
         <is>
-          <t>Same objects as last year's Art Sales layout</t>
+          <t>2022–2024 lots stay. 2025 adds Roman Gold Belt SALE and Venus joint SALE (EPGC share).</t>
         </is>
       </c>
       <c r="E27" s="226" t="inlineStr">
@@ -9445,12 +9459,12 @@
     <row r="34">
       <c r="A34" s="224" t="inlineStr">
         <is>
-          <t>Dump EOEB $130,270 or L5 $87,396.32 onto P&amp;L</t>
+          <t>Dump EOEB $130,270 or other L5 $37,396.32 onto P&amp;L</t>
         </is>
       </c>
       <c r="B34" s="224" t="inlineStr">
         <is>
-          <t>Mixed art + consultant. Invoice split still ASK.</t>
+          <t>Mixed art + consultant. Invoice split still ASK. Belt $50k is locked SALE; remaining L5 is not.</t>
         </is>
       </c>
       <c r="C34" s="224" t="inlineStr"/>
@@ -9606,7 +9620,7 @@
     <row r="43">
       <c r="A43" s="229" t="inlineStr">
         <is>
-          <t>EPGC Art Sales vs $150,000</t>
+          <t>EPGC Art Sales vs $226,000</t>
         </is>
       </c>
       <c r="B43" s="230">
@@ -9614,7 +9628,7 @@
         <v/>
       </c>
       <c r="C43" s="230" t="n">
-        <v>150000</v>
+        <v>226000</v>
       </c>
       <c r="D43" s="229">
         <f>IF(ROUND(B43,2)=ROUND(C43,2),"MATCH","FAIL")</f>
@@ -9654,6 +9668,144 @@
           <t>Color key: peach = entered like last year. Green = locked from bank or user. Yellow = WAIT (statement or Cost). Not tax advice.</t>
         </is>
       </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="238" t="inlineStr">
+        <is>
+          <t>DEAL CLASSIFIER (conceptual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="238" t="inlineStr">
+        <is>
+          <t>Classifier</t>
+        </is>
+      </c>
+      <c r="B49" s="238" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C49" s="238" t="inlineStr">
+        <is>
+          <t>2025 locked example</t>
+        </is>
+      </c>
+      <c r="D49" s="238" t="inlineStr">
+        <is>
+          <t>Still ASK / unallocated</t>
+        </is>
+      </c>
+      <c r="E49" s="238" t="inlineStr"/>
+    </row>
+    <row r="50" ht="32" customHeight="1" s="137">
+      <c r="A50" s="208" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="B50" s="208" t="inlineStr">
+        <is>
+          <t>Art object sold; Art Sales register + EPGC Art Sales gross cash; I8 gets NET if Cost known</t>
+        </is>
+      </c>
+      <c r="C50" s="208" t="inlineStr">
+        <is>
+          <t>Roman Gold Belt L5 $50,000 / Cost $45,000</t>
+        </is>
+      </c>
+      <c r="D50" s="208" t="inlineStr"/>
+    </row>
+    <row r="51" ht="32" customHeight="1" s="137">
+      <c r="A51" s="208" t="inlineStr">
+        <is>
+          <t>SALE (joint, EPGC share)</t>
+        </is>
+      </c>
+      <c r="B51" s="208" t="inlineStr">
+        <is>
+          <t>Joint purchase; register Sale Price = EPGC proceeds, not full hammer</t>
+        </is>
+      </c>
+      <c r="C51" s="208" t="inlineStr">
+        <is>
+          <t>Venus Erdal remittance $26,000 / EPGC Cost $20,000</t>
+        </is>
+      </c>
+      <c r="D51" s="208" t="inlineStr"/>
+    </row>
+    <row r="52" ht="32" customHeight="1" s="137">
+      <c r="A52" s="208" t="inlineStr">
+        <is>
+          <t>FEE</t>
+        </is>
+      </c>
+      <c r="B52" s="208" t="inlineStr">
+        <is>
+          <t>Advisory / consultant income or expertise expense — never I8</t>
+        </is>
+      </c>
+      <c r="C52" s="208" t="inlineStr">
+        <is>
+          <t>David Aaron June $13,595 Consultant; Wise write-ups $992.80 Fees</t>
+        </is>
+      </c>
+      <c r="D52" s="208" t="inlineStr"/>
+    </row>
+    <row r="53" ht="32" customHeight="1" s="137">
+      <c r="A53" s="208" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B53" s="208" t="inlineStr">
+        <is>
+          <t>In and out, not P&amp;L</t>
+        </is>
+      </c>
+      <c r="C53" s="208" t="inlineStr">
+        <is>
+          <t>Koziol $150,000 10/20 → Ariadne $150,000 10/21</t>
+        </is>
+      </c>
+      <c r="D53" s="208" t="inlineStr"/>
+    </row>
+    <row r="54" ht="32" customHeight="1" s="137">
+      <c r="A54" s="190" t="inlineStr">
+        <is>
+          <t>INVENTORY</t>
+        </is>
+      </c>
+      <c r="B54" s="190" t="inlineStr">
+        <is>
+          <t>Named or unnamed purchase still unsold</t>
+        </is>
+      </c>
+      <c r="C54" s="190" t="inlineStr">
+        <is>
+          <t>Fortuna Aug unnamed $20,000</t>
+        </is>
+      </c>
+      <c r="D54" s="190" t="inlineStr"/>
+    </row>
+    <row r="55" ht="32" customHeight="1" s="137">
+      <c r="A55" s="190" t="inlineStr">
+        <is>
+          <t>UNALLOCATED</t>
+        </is>
+      </c>
+      <c r="B55" s="190" t="inlineStr">
+        <is>
+          <t>Mixed pattern confirmed; invoice-level split still ASK; do not dump</t>
+        </is>
+      </c>
+      <c r="C55" s="190" t="inlineStr">
+        <is>
+          <t>EOEB remainder $130,270.00; other L5 $37,396.32; other Erdal IN $31,000; Aysel $50,000</t>
+        </is>
+      </c>
+      <c r="D55" s="190" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -23249,8 +23401,8 @@
       <c r="G53" s="179" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="179" t="n">
-        <v>0</v>
+      <c r="H53" s="183" t="n">
+        <v>76000</v>
       </c>
       <c r="I53" s="179" t="n">
         <v>0</v>
@@ -24051,7 +24203,7 @@
     <row r="75" ht="72" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-20: Art Sales = MATCHED/LOCKED cash (Berk $14,000 Jan + Berk $30,000 / mosaics $105,000 / Aquinas books $1,000 Feb = $150,000). Consultant June $13,595 = David Aaron Limited LOCKED (user: consultant fee, not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270.00 and L5 $87,396.32 MIXED PATTERN CONFIRMED (art sales + advisory/consultant) — invoice-level split still ASK; not dumped onto Consultant or Art Sales. Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments, not this tab. Newstar $23,581 is Art Sales COGS, not operating expense. Dec Wise $565.75 reimbursed — not on Consultant Fees. Aquinas books Cost TBD — cash on Art Sales, not in I8. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) = $226,000. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 and other L5 $37,396.32 MIXED PATTERN CONFIRMED — invoice-level split still ASK; not dumped. Other Erdal IN 10/9 $25,000 and 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Fortuna Aug unnamed $20,000 still ASK (not Venus, not belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD — cash on Art Sales, not in I8. Venus Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -27600,7 +27752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z134"/>
+  <dimension ref="A1:Z135"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="47.86" customWidth="1" style="137" min="1" max="1"/>
@@ -27617,6 +27769,11 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="137">
+      <c r="A1" s="234" t="inlineStr">
+        <is>
+          <t>Art Sales and Purchases</t>
+        </is>
+      </c>
       <c r="B1" s="104" t="n"/>
       <c r="C1" s="88" t="n"/>
       <c r="F1" s="88" t="n"/>
@@ -27688,6 +27845,11 @@
           <t xml:space="preserve">Days in Inventory </t>
         </is>
       </c>
+      <c r="K3" s="234" t="inlineStr">
+        <is>
+          <t>Classifier</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="137">
       <c r="A4" s="122" t="inlineStr">
@@ -28186,6 +28348,11 @@
         </is>
       </c>
       <c r="I16" s="105" t="n"/>
+      <c r="K16" s="234" t="inlineStr">
+        <is>
+          <t>Classifier</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="14.25" customHeight="1" s="137">
       <c r="A17" s="122" t="inlineStr">
@@ -29094,6 +29261,11 @@
         </is>
       </c>
       <c r="I39" s="105" t="n"/>
+      <c r="K39" s="234" t="inlineStr">
+        <is>
+          <t>Classifier</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="137">
       <c r="A40" s="122" t="inlineStr">
@@ -29444,6 +29616,11 @@
         </is>
       </c>
       <c r="I50" s="105" t="n"/>
+      <c r="K50" s="234" t="inlineStr">
+        <is>
+          <t>Classifier</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="137">
       <c r="A51" s="113" t="inlineStr">
@@ -30308,212 +30485,260 @@
       </c>
     </row>
     <row r="78" ht="48" customHeight="1" s="137">
-      <c r="A78" s="178" t="inlineStr">
+      <c r="A78" s="181" t="inlineStr">
+        <is>
+          <t>Roman Gold Belt</t>
+        </is>
+      </c>
+      <c r="B78" s="181" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere</t>
+        </is>
+      </c>
+      <c r="C78" s="183" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D78" s="209" t="n">
+        <v>45859</v>
+      </c>
+      <c r="E78" s="181" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="F78" s="183" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G78" s="209" t="n">
+        <v>45853</v>
+      </c>
+      <c r="H78" s="183">
+        <f>F78-C78</f>
+        <v/>
+      </c>
+      <c r="I78" s="208" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 SALE. Bought Fortuna/Erdal Dere 7/21 −$45,000 (Mercury 8291 native memo: Roman Gold Belt). Sold to L5. Working sale: L5 7/15 +$50,000 (only L5 payment large enough; L5 paid 6 days before Fortuna Cost — back-to-back dealer cash). Net $5,000. Do NOT attach remaining L5 invoices. Classifier: SALE. Not unsold inventory. Not consultant. Not pass-through. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="J78" s="181" t="n"/>
+      <c r="K78" s="181" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="60" customHeight="1" s="137">
+      <c r="A79" s="181" t="inlineStr">
+        <is>
+          <t>Bronze head of a goddess, likely Venus (joint; EPGC share)</t>
+        </is>
+      </c>
+      <c r="B79" s="181" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere</t>
+        </is>
+      </c>
+      <c r="C79" s="183" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D79" s="209" t="n">
+        <v>45786</v>
+      </c>
+      <c r="E79" s="181" t="inlineStr">
+        <is>
+          <t>Erdal Dere</t>
+        </is>
+      </c>
+      <c r="F79" s="183" t="n">
+        <v>26000</v>
+      </c>
+      <c r="G79" s="209" t="n">
+        <v>45862</v>
+      </c>
+      <c r="H79" s="183">
+        <f>F79-C79</f>
+        <v/>
+      </c>
+      <c r="I79" s="208" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 joint SALE (EPGC share). Erdal and Jacob bought together. EPGC Cost: Fortuna 5/9 −$20,000 (native memo: bronze head of a goddess, likely Venus). Erdal sold it and paid back Jacob’s investment plus earnings. Working remittance: Erdal Dere IN 7/24 +$26,000 = $20,000 investment + $6,000 earnings. Sale Price on this register is EPGC proceeds ($26,000), not the object’s full hammer. Classifier: SALE (joint, EPGC share). Not unsold inventory. Not consultant. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="J79" s="181" t="n"/>
+      <c r="K79" s="181" t="inlineStr">
+        <is>
+          <t>SALE (joint, EPGC share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="14.25" customHeight="1" s="137">
+      <c r="A80" s="184" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H78" s="138">
-        <f>SUM(H51:H75)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" ht="48" customHeight="1" s="137">
-      <c r="A79" s="210" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Newstar $23,581 is jewelry fabrication COGS, parked below — not in sold-lot Cost (Berk gem/scarab lots already sold in February). David Aaron $13,595 (6/24) is LOCKED consultant fee — not a sale (EPGC Consultant June). Aquinas Hobor $1,000 (2/4) is LOCKED book sale — EPGC Art Sales February; Cost TBD (not in I8). Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="14.25" customHeight="1" s="137">
-      <c r="A80" s="119" t="inlineStr">
+      <c r="H80" s="235">
+        <f>SUM(H51:H75)+H78+H79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" ht="64" customHeight="1" s="137">
+      <c r="A81" s="208" t="inlineStr">
+        <is>
+          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000 (Sale Price = remittance, not full hammer). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 or other L5 $37,396.32. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="14.25" customHeight="1" s="137">
+      <c r="A82" s="119" t="inlineStr">
         <is>
           <t>Art Purchases/Inventory</t>
         </is>
       </c>
-      <c r="B80" s="120" t="n"/>
-      <c r="C80" s="100" t="n"/>
-      <c r="D80" s="101" t="n"/>
-      <c r="E80" s="99" t="n"/>
-      <c r="F80" s="100" t="n"/>
-      <c r="G80" s="101" t="n"/>
-      <c r="H80" s="99" t="n"/>
-      <c r="I80" s="121" t="n"/>
-      <c r="J80" s="99" t="n"/>
-      <c r="K80" s="99" t="n"/>
-      <c r="L80" s="99" t="n"/>
-      <c r="M80" s="99" t="n"/>
-      <c r="N80" s="99" t="n"/>
-      <c r="O80" s="99" t="n"/>
-      <c r="P80" s="99" t="n"/>
-      <c r="Q80" s="99" t="n"/>
-      <c r="R80" s="99" t="n"/>
-      <c r="S80" s="99" t="n"/>
-      <c r="T80" s="99" t="n"/>
-      <c r="U80" s="99" t="n"/>
-      <c r="V80" s="99" t="n"/>
-      <c r="W80" s="99" t="n"/>
-      <c r="X80" s="99" t="n"/>
-      <c r="Y80" s="99" t="n"/>
-      <c r="Z80" s="99" t="n"/>
-    </row>
-    <row r="81" ht="14.25" customHeight="1" s="137">
-      <c r="A81" s="122" t="inlineStr">
-        <is>
-          <t>30 Paleothic and Neolithic Stone Tools</t>
-        </is>
-      </c>
-      <c r="B81" s="116" t="inlineStr">
-        <is>
-          <t>Holestein</t>
-        </is>
-      </c>
-      <c r="C81" s="88" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E81" s="105" t="n"/>
-    </row>
-    <row r="82" ht="14.25" customHeight="1" s="137">
-      <c r="A82" s="122" t="inlineStr">
-        <is>
-          <t>A Tairona Figure</t>
-        </is>
-      </c>
-      <c r="B82" s="116" t="inlineStr">
-        <is>
-          <t>Live Auctioneers</t>
-        </is>
-      </c>
-      <c r="C82" s="88" t="n">
-        <v>250</v>
-      </c>
-      <c r="D82" s="92" t="n">
-        <v>45119</v>
-      </c>
-      <c r="E82" s="105" t="n"/>
+      <c r="B82" s="120" t="n"/>
+      <c r="C82" s="100" t="n"/>
+      <c r="D82" s="101" t="n"/>
+      <c r="E82" s="99" t="n"/>
+      <c r="F82" s="100" t="n"/>
+      <c r="G82" s="101" t="n"/>
+      <c r="H82" s="99" t="n"/>
+      <c r="I82" s="121" t="n"/>
+      <c r="J82" s="99" t="n"/>
+      <c r="K82" s="99" t="n"/>
+      <c r="L82" s="99" t="n"/>
+      <c r="M82" s="99" t="n"/>
+      <c r="N82" s="99" t="n"/>
+      <c r="O82" s="99" t="n"/>
+      <c r="P82" s="99" t="n"/>
+      <c r="Q82" s="99" t="n"/>
+      <c r="R82" s="99" t="n"/>
+      <c r="S82" s="99" t="n"/>
+      <c r="T82" s="99" t="n"/>
+      <c r="U82" s="99" t="n"/>
+      <c r="V82" s="99" t="n"/>
+      <c r="W82" s="99" t="n"/>
+      <c r="X82" s="99" t="n"/>
+      <c r="Y82" s="99" t="n"/>
+      <c r="Z82" s="99" t="n"/>
     </row>
     <row r="83" ht="14.25" customHeight="1" s="137">
       <c r="A83" s="122" t="inlineStr">
         <is>
-          <t>A Tairona Figure</t>
+          <t>30 Paleothic and Neolithic Stone Tools</t>
         </is>
       </c>
       <c r="B83" s="116" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Holestein</t>
         </is>
       </c>
       <c r="C83" s="88" t="n">
-        <v>300</v>
-      </c>
-      <c r="D83" s="92" t="n">
-        <v>45119</v>
+        <v>4000</v>
       </c>
       <c r="E83" s="105" t="n"/>
     </row>
     <row r="84" ht="14.25" customHeight="1" s="137">
       <c r="A84" s="122" t="inlineStr">
         <is>
-          <t>A Pair of Greek Bronze Greeves</t>
+          <t>A Tairona Figure</t>
         </is>
       </c>
       <c r="B84" s="116" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C84" s="88" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="D84" s="92" t="n">
-        <v>45145</v>
+        <v>45119</v>
       </c>
       <c r="E84" s="105" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1" s="137">
       <c r="A85" s="122" t="inlineStr">
         <is>
-          <t>An Illyrian Bronze Helmet</t>
+          <t>A Tairona Figure</t>
         </is>
       </c>
       <c r="B85" s="116" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C85" s="88" t="n">
-        <v>551.25</v>
+        <v>300</v>
       </c>
       <c r="D85" s="92" t="n">
-        <v>45114</v>
+        <v>45119</v>
       </c>
       <c r="E85" s="105" t="n"/>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="137">
       <c r="A86" s="122" t="inlineStr">
         <is>
-          <t>An Egyptian Faience Ibis</t>
-        </is>
-      </c>
-      <c r="B86" s="104" t="inlineStr">
-        <is>
-          <t>Hindman</t>
+          <t>A Pair of Greek Bronze Greeves</t>
+        </is>
+      </c>
+      <c r="B86" s="116" t="inlineStr">
+        <is>
+          <t>ebay</t>
         </is>
       </c>
       <c r="C86" s="88" t="n">
-        <v>375</v>
+        <v>200</v>
       </c>
       <c r="D86" s="92" t="n">
-        <v>44343</v>
-      </c>
-      <c r="E86" s="92" t="n"/>
-      <c r="F86" s="88" t="n"/>
-      <c r="I86" s="105" t="n"/>
+        <v>45145</v>
+      </c>
+      <c r="E86" s="105" t="n"/>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="137">
       <c r="A87" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
-        </is>
-      </c>
-      <c r="B87" s="104" t="inlineStr">
-        <is>
-          <t>Live Auctioneers</t>
+          <t>An Illyrian Bronze Helmet</t>
+        </is>
+      </c>
+      <c r="B87" s="116" t="inlineStr">
+        <is>
+          <t>ebay</t>
         </is>
       </c>
       <c r="C87" s="88" t="n">
-        <v>293</v>
+        <v>551.25</v>
       </c>
       <c r="D87" s="92" t="n">
-        <v>44548</v>
-      </c>
-      <c r="F87" s="88" t="n"/>
-      <c r="I87" s="105" t="n"/>
+        <v>45114</v>
+      </c>
+      <c r="E87" s="105" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="137">
       <c r="A88" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
+          <t>An Egyptian Faience Ibis</t>
         </is>
       </c>
       <c r="B88" s="104" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C88" s="88" t="n">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="D88" s="92" t="n">
-        <v>44548</v>
-      </c>
+        <v>44343</v>
+      </c>
+      <c r="E88" s="92" t="n"/>
       <c r="F88" s="88" t="n"/>
       <c r="I88" s="105" t="n"/>
     </row>
     <row r="89" ht="14.25" customHeight="1" s="137">
       <c r="A89" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
         </is>
       </c>
       <c r="B89" s="104" t="inlineStr">
@@ -30533,19 +30758,19 @@
     <row r="90" ht="14.25" customHeight="1" s="137">
       <c r="A90" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
         </is>
       </c>
       <c r="B90" s="104" t="inlineStr">
         <is>
-          <t>Pace African Art</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C90" s="88" t="n">
-        <v>1000</v>
+        <v>293</v>
       </c>
       <c r="D90" s="92" t="n">
-        <v>44562</v>
+        <v>44548</v>
       </c>
       <c r="F90" s="88" t="n"/>
       <c r="I90" s="105" t="n"/>
@@ -30553,16 +30778,19 @@
     <row r="91" ht="14.25" customHeight="1" s="137">
       <c r="A91" s="122" t="inlineStr">
         <is>
-          <t>Carved Ostrish Egg</t>
+          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
         </is>
       </c>
       <c r="B91" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etsy </t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C91" s="88" t="n">
-        <v>90</v>
+        <v>293</v>
+      </c>
+      <c r="D91" s="92" t="n">
+        <v>44548</v>
       </c>
       <c r="F91" s="88" t="n"/>
       <c r="I91" s="105" t="n"/>
@@ -30570,16 +30798,19 @@
     <row r="92" ht="14.25" customHeight="1" s="137">
       <c r="A92" s="122" t="inlineStr">
         <is>
-          <t>Carved Goose Egg</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B92" s="104" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>Pace African Art</t>
         </is>
       </c>
       <c r="C92" s="88" t="n">
-        <v>30</v>
+        <v>1000</v>
+      </c>
+      <c r="D92" s="92" t="n">
+        <v>44562</v>
       </c>
       <c r="F92" s="88" t="n"/>
       <c r="I92" s="105" t="n"/>
@@ -30587,16 +30818,16 @@
     <row r="93" ht="14.25" customHeight="1" s="137">
       <c r="A93" s="122" t="inlineStr">
         <is>
-          <t>Carved Goose Egg</t>
+          <t>Carved Ostrish Egg</t>
         </is>
       </c>
       <c r="B93" s="104" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t xml:space="preserve">Etsy </t>
         </is>
       </c>
       <c r="C93" s="88" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="F93" s="88" t="n"/>
       <c r="I93" s="105" t="n"/>
@@ -30604,97 +30835,91 @@
     <row r="94" ht="14.25" customHeight="1" s="137">
       <c r="A94" s="122" t="inlineStr">
         <is>
-          <t>Quimbaya Figure (Gift)</t>
+          <t>Carved Goose Egg</t>
         </is>
       </c>
       <c r="B94" s="104" t="inlineStr">
         <is>
-          <t>Jeffrey Norris</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C94" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="D94" s="92" t="n">
-        <v>45079</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F94" s="88" t="n"/>
       <c r="I94" s="105" t="n"/>
     </row>
     <row r="95" ht="14.25" customHeight="1" s="137">
       <c r="A95" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal (Gift)</t>
+          <t>Carved Goose Egg</t>
         </is>
       </c>
       <c r="B95" s="104" t="inlineStr">
         <is>
-          <t>Aquinas Hobor</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C95" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="D95" s="92" t="n">
-        <v>45079</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F95" s="88" t="n"/>
       <c r="I95" s="105" t="n"/>
     </row>
     <row r="96" ht="14.25" customHeight="1" s="137">
       <c r="A96" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>Quimbaya Figure (Gift)</t>
         </is>
       </c>
       <c r="B96" s="104" t="inlineStr">
         <is>
-          <t>Aquinas Hobor</t>
-        </is>
-      </c>
-      <c r="C96" s="103" t="n">
-        <v>500</v>
+          <t>Jeffrey Norris</t>
+        </is>
+      </c>
+      <c r="C96" s="88" t="n">
+        <v>10</v>
       </c>
       <c r="D96" s="92" t="n">
         <v>45079</v>
       </c>
-      <c r="F96" s="88" t="n"/>
       <c r="I96" s="105" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1" s="137">
       <c r="A97" s="122" t="inlineStr">
         <is>
-          <t>Two Songye and Bozo Vessels</t>
+          <t>A Saharan Stone Discoidal (Gift)</t>
         </is>
       </c>
       <c r="B97" s="104" t="inlineStr">
         <is>
-          <t>Hindman</t>
-        </is>
-      </c>
-      <c r="C97" s="103" t="n">
-        <v>138.91</v>
+          <t>Aquinas Hobor</t>
+        </is>
+      </c>
+      <c r="C97" s="88" t="n">
+        <v>10</v>
       </c>
       <c r="D97" s="92" t="n">
-        <v>45211</v>
-      </c>
-      <c r="F97" s="88" t="n"/>
+        <v>45079</v>
+      </c>
       <c r="I97" s="105" t="n"/>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="137">
       <c r="A98" s="122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sword 9th Century </t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B98" s="104" t="inlineStr">
         <is>
-          <t>Zevantiques</t>
+          <t>Aquinas Hobor</t>
         </is>
       </c>
       <c r="C98" s="103" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="D98" s="92" t="n">
-        <v>45311</v>
+        <v>45079</v>
       </c>
       <c r="F98" s="88" t="n"/>
       <c r="I98" s="105" t="n"/>
@@ -30702,19 +30927,19 @@
     <row r="99" ht="14.25" customHeight="1" s="137">
       <c r="A99" s="122" t="inlineStr">
         <is>
-          <t>A Roman Marble Plaque with Insciption</t>
+          <t>Two Songye and Bozo Vessels</t>
         </is>
       </c>
       <c r="B99" s="104" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C99" s="103" t="n">
-        <v>1331.41</v>
+        <v>138.91</v>
       </c>
       <c r="D99" s="92" t="n">
-        <v>45546</v>
+        <v>45211</v>
       </c>
       <c r="F99" s="88" t="n"/>
       <c r="I99" s="105" t="n"/>
@@ -30722,105 +30947,123 @@
     <row r="100" ht="14.25" customHeight="1" s="137">
       <c r="A100" s="122" t="inlineStr">
         <is>
-          <t>Erotic Intaglio Finger Ring</t>
+          <t xml:space="preserve">Sword 9th Century </t>
         </is>
       </c>
       <c r="B100" s="104" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Zevantiques</t>
         </is>
       </c>
       <c r="C100" s="103" t="n">
-        <v>205.07</v>
+        <v>3000</v>
       </c>
       <c r="D100" s="92" t="n">
-        <v>45446</v>
+        <v>45311</v>
       </c>
       <c r="F100" s="88" t="n"/>
       <c r="I100" s="105" t="n"/>
     </row>
     <row r="101" ht="14.25" customHeight="1" s="137">
-      <c r="B101" s="104" t="n"/>
-      <c r="C101" s="103" t="n"/>
-      <c r="D101" s="92" t="n"/>
+      <c r="A101" s="122" t="inlineStr">
+        <is>
+          <t>A Roman Marble Plaque with Insciption</t>
+        </is>
+      </c>
+      <c r="B101" s="104" t="inlineStr">
+        <is>
+          <t>ebay</t>
+        </is>
+      </c>
+      <c r="C101" s="103" t="n">
+        <v>1331.41</v>
+      </c>
+      <c r="D101" s="92" t="n">
+        <v>45546</v>
+      </c>
       <c r="F101" s="88" t="n"/>
       <c r="I101" s="105" t="n"/>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="137">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B102" s="104" t="n"/>
-      <c r="C102" s="86" t="n"/>
+      <c r="A102" s="122" t="inlineStr">
+        <is>
+          <t>Erotic Intaglio Finger Ring</t>
+        </is>
+      </c>
+      <c r="B102" s="104" t="inlineStr">
+        <is>
+          <t>ebay</t>
+        </is>
+      </c>
+      <c r="C102" s="103" t="n">
+        <v>205.07</v>
+      </c>
+      <c r="D102" s="92" t="n">
+        <v>45446</v>
+      </c>
       <c r="F102" s="88" t="n"/>
       <c r="I102" s="105" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="137">
       <c r="B103" s="104" t="n"/>
-      <c r="C103" s="88" t="n"/>
+      <c r="C103" s="103" t="n"/>
+      <c r="D103" s="92" t="n"/>
       <c r="F103" s="88" t="n"/>
       <c r="I103" s="105" t="n"/>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="137">
-      <c r="A104" s="119" t="inlineStr">
-        <is>
-          <t>Office/Business Inventory</t>
-        </is>
-      </c>
-      <c r="B104" s="120" t="n"/>
-      <c r="C104" s="100" t="n"/>
-      <c r="D104" s="99" t="n"/>
-      <c r="E104" s="99" t="n"/>
-      <c r="F104" s="100" t="n"/>
-      <c r="G104" s="99" t="n"/>
-      <c r="H104" s="99" t="n"/>
-      <c r="I104" s="121" t="n"/>
-      <c r="J104" s="99" t="n"/>
-      <c r="K104" s="99" t="n"/>
-      <c r="L104" s="99" t="n"/>
-      <c r="M104" s="99" t="n"/>
-      <c r="N104" s="99" t="n"/>
-      <c r="O104" s="99" t="n"/>
-      <c r="P104" s="99" t="n"/>
-      <c r="Q104" s="99" t="n"/>
-      <c r="R104" s="99" t="n"/>
-      <c r="S104" s="99" t="n"/>
-      <c r="T104" s="99" t="n"/>
-      <c r="U104" s="99" t="n"/>
-      <c r="V104" s="99" t="n"/>
-      <c r="W104" s="99" t="n"/>
-      <c r="X104" s="99" t="n"/>
-      <c r="Y104" s="99" t="n"/>
-      <c r="Z104" s="99" t="n"/>
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B104" s="104" t="n"/>
+      <c r="C104" s="86" t="n"/>
+      <c r="F104" s="88" t="n"/>
+      <c r="I104" s="105" t="n"/>
     </row>
     <row r="105" ht="14.25" customHeight="1" s="137">
-      <c r="A105" s="122" t="inlineStr">
-        <is>
-          <t>Sofa</t>
-        </is>
-      </c>
       <c r="B105" s="104" t="n"/>
       <c r="C105" s="88" t="n"/>
       <c r="F105" s="88" t="n"/>
       <c r="I105" s="105" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="137">
-      <c r="A106" s="122" t="inlineStr">
-        <is>
-          <t>Space Heater</t>
-        </is>
-      </c>
-      <c r="B106" s="104" t="n"/>
-      <c r="C106" s="88" t="n"/>
-      <c r="F106" s="88" t="n"/>
-      <c r="I106" s="105" t="n"/>
+      <c r="A106" s="119" t="inlineStr">
+        <is>
+          <t>Office/Business Inventory</t>
+        </is>
+      </c>
+      <c r="B106" s="120" t="n"/>
+      <c r="C106" s="100" t="n"/>
+      <c r="D106" s="99" t="n"/>
+      <c r="E106" s="99" t="n"/>
+      <c r="F106" s="100" t="n"/>
+      <c r="G106" s="99" t="n"/>
+      <c r="H106" s="99" t="n"/>
+      <c r="I106" s="121" t="n"/>
+      <c r="J106" s="99" t="n"/>
+      <c r="K106" s="99" t="n"/>
+      <c r="L106" s="99" t="n"/>
+      <c r="M106" s="99" t="n"/>
+      <c r="N106" s="99" t="n"/>
+      <c r="O106" s="99" t="n"/>
+      <c r="P106" s="99" t="n"/>
+      <c r="Q106" s="99" t="n"/>
+      <c r="R106" s="99" t="n"/>
+      <c r="S106" s="99" t="n"/>
+      <c r="T106" s="99" t="n"/>
+      <c r="U106" s="99" t="n"/>
+      <c r="V106" s="99" t="n"/>
+      <c r="W106" s="99" t="n"/>
+      <c r="X106" s="99" t="n"/>
+      <c r="Y106" s="99" t="n"/>
+      <c r="Z106" s="99" t="n"/>
     </row>
     <row r="107" ht="14.25" customHeight="1" s="137">
       <c r="A107" s="122" t="inlineStr">
         <is>
-          <t>Shelving</t>
+          <t>Sofa</t>
         </is>
       </c>
       <c r="B107" s="104" t="n"/>
@@ -30831,7 +31074,7 @@
     <row r="108" ht="14.25" customHeight="1" s="137">
       <c r="A108" s="122" t="inlineStr">
         <is>
-          <t>Storage Bins</t>
+          <t>Space Heater</t>
         </is>
       </c>
       <c r="B108" s="104" t="n"/>
@@ -30842,7 +31085,7 @@
     <row r="109" ht="14.25" customHeight="1" s="137">
       <c r="A109" s="122" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Shelving</t>
         </is>
       </c>
       <c r="B109" s="104" t="n"/>
@@ -30853,7 +31096,7 @@
     <row r="110" ht="14.25" customHeight="1" s="137">
       <c r="A110" s="122" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Storage Bins</t>
         </is>
       </c>
       <c r="B110" s="104" t="n"/>
@@ -30864,7 +31107,7 @@
     <row r="111" ht="14.25" customHeight="1" s="137">
       <c r="A111" s="122" t="inlineStr">
         <is>
-          <t>Art Library</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="B111" s="104" t="n"/>
@@ -30875,7 +31118,7 @@
     <row r="112" ht="14.25" customHeight="1" s="137">
       <c r="A112" s="122" t="inlineStr">
         <is>
-          <t>Standing Desk</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B112" s="104" t="n"/>
@@ -30884,15 +31127,20 @@
       <c r="I112" s="105" t="n"/>
     </row>
     <row r="113" ht="14.25" customHeight="1" s="137">
+      <c r="A113" s="122" t="inlineStr">
+        <is>
+          <t>Art Library</t>
+        </is>
+      </c>
       <c r="B113" s="104" t="n"/>
       <c r="C113" s="88" t="n"/>
       <c r="F113" s="88" t="n"/>
       <c r="I113" s="105" t="n"/>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="137">
-      <c r="A114" s="156" t="inlineStr">
-        <is>
-          <t>2025 CC inventory (not in Cost total until object is named)</t>
+      <c r="A114" s="122" t="inlineStr">
+        <is>
+          <t>Standing Desk</t>
         </is>
       </c>
       <c r="B114" s="104" t="n"/>
@@ -30901,49 +31149,26 @@
       <c r="I114" s="105" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="137">
-      <c r="A115" s="0" t="inlineStr">
-        <is>
-          <t>Los Angeles Modern Auctions (inventory purchase)</t>
-        </is>
-      </c>
-      <c r="B115" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C115" s="157" t="n">
-        <v>6821.06</v>
-      </c>
-      <c r="D115" s="0" t="inlineStr">
-        <is>
-          <t>2025-07-24</t>
-        </is>
-      </c>
+      <c r="B115" s="104" t="n"/>
+      <c r="C115" s="88" t="n"/>
+      <c r="F115" s="88" t="n"/>
+      <c r="I115" s="105" t="n"/>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="137">
-      <c r="A116" s="0" t="inlineStr">
-        <is>
-          <t>Hindman LLC (inventory purchase)</t>
-        </is>
-      </c>
-      <c r="B116" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C116" s="157" t="n">
-        <v>282.24</v>
-      </c>
-      <c r="D116" s="0" t="inlineStr">
-        <is>
-          <t>2025-04-03</t>
-        </is>
-      </c>
+      <c r="A116" s="156" t="inlineStr">
+        <is>
+          <t>2025 CC inventory (not in Cost total until object is named)</t>
+        </is>
+      </c>
+      <c r="B116" s="104" t="n"/>
+      <c r="C116" s="88" t="n"/>
+      <c r="F116" s="88" t="n"/>
+      <c r="I116" s="105" t="n"/>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="137">
       <c r="A117" s="0" t="inlineStr">
         <is>
-          <t>Hindman LLC (inventory purchase)</t>
+          <t>Los Angeles Modern Auctions (inventory purchase)</t>
         </is>
       </c>
       <c r="B117" s="0" t="inlineStr">
@@ -30952,254 +31177,279 @@
         </is>
       </c>
       <c r="C117" s="157" t="n">
-        <v>403.51</v>
+        <v>6821.06</v>
       </c>
       <c r="D117" s="0" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-07-24</t>
         </is>
       </c>
     </row>
     <row r="118" ht="14.25" customHeight="1" s="137">
       <c r="A118" s="0" t="inlineStr">
         <is>
+          <t>Hindman LLC (inventory purchase)</t>
+        </is>
+      </c>
+      <c r="B118" s="0" t="inlineStr">
+        <is>
+          <t>Sapphire 5423</t>
+        </is>
+      </c>
+      <c r="C118" s="157" t="n">
+        <v>282.24</v>
+      </c>
+      <c r="D118" s="0" t="inlineStr">
+        <is>
+          <t>2025-04-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="14.25" customHeight="1" s="137">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t>Hindman LLC (inventory purchase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="14.25" customHeight="1" s="137">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
           <t>The Great Frame Up (inventory framing)</t>
         </is>
       </c>
-      <c r="B118" s="0" t="inlineStr">
+      <c r="B120" s="0" t="inlineStr">
         <is>
           <t>Sapphire 5423</t>
         </is>
       </c>
-      <c r="C118" s="157" t="n">
+      <c r="C120" s="157" t="n">
         <v>536.41</v>
       </c>
-      <c r="D118" s="0" t="inlineStr">
+      <c r="D120" s="0" t="inlineStr">
         <is>
           <t>2025-02-16</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="14.25" customHeight="1" s="137"/>
-    <row r="120" ht="14.25" customHeight="1" s="137">
-      <c r="A120" s="201" t="inlineStr">
+    <row r="121" ht="14.25" customHeight="1" s="137"/>
+    <row r="122" ht="14.25" customHeight="1" s="137">
+      <c r="A122" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury 8291 — David Aaron Limited is LOCKED consultant fee (not Art Sales)</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="14.25" customHeight="1" s="137">
-      <c r="A121" s="181" t="inlineStr">
+    <row r="123" ht="14.25" customHeight="1" s="137">
+      <c r="A123" s="181" t="inlineStr">
         <is>
           <t>NOT a 2025 art sale — David Aaron Limited consultant fee (EPGC Consultant June)</t>
         </is>
       </c>
-      <c r="B121" s="181" t="inlineStr">
+      <c r="B123" s="181" t="inlineStr">
         <is>
           <t>David Aaron Limited</t>
         </is>
       </c>
-      <c r="C121" s="181" t="n"/>
-      <c r="D121" s="181" t="n"/>
-      <c r="E121" s="181" t="n"/>
-      <c r="F121" s="183" t="n"/>
-      <c r="G121" s="206" t="n"/>
-      <c r="H121" s="206" t="n"/>
-      <c r="I121" s="181" t="inlineStr">
+      <c r="C123" s="181" t="n"/>
+      <c r="D123" s="181" t="n"/>
+      <c r="E123" s="181" t="n"/>
+      <c r="F123" s="183" t="n"/>
+      <c r="G123" s="206" t="n"/>
+      <c r="H123" s="206" t="n"/>
+      <c r="I123" s="181" t="inlineStr">
         <is>
           <t>LOCKED 2026-09-20: consultant fee, not a sale. $13,595 is on EPGC Consultant June. Not tax advice.</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="14.25" customHeight="1" s="137"/>
-    <row r="123" ht="14.25" customHeight="1" s="137">
-      <c r="A123" s="201" t="inlineStr">
+    <row r="124" ht="14.25" customHeight="1" s="137"/>
+    <row r="125" ht="14.25" customHeight="1" s="137">
+      <c r="A125" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury COGS — Newstar Jewelers (LOCKED jewelry fabrication)</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="14.25" customHeight="1" s="137">
-      <c r="A124" s="202" t="inlineStr">
-        <is>
-          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
-        </is>
-      </c>
-      <c r="B124" s="202" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C124" s="203" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D124" s="202" t="inlineStr">
-        <is>
-          <t>2025-10-14</t>
-        </is>
-      </c>
-      <c r="I124" s="0" t="inlineStr">
-        <is>
-          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="14.25" customHeight="1" s="137">
-      <c r="A125" s="202" t="inlineStr">
-        <is>
-          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
-        </is>
-      </c>
-      <c r="B125" s="202" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C125" s="203" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D125" s="202" t="inlineStr">
-        <is>
-          <t>2025-11-12</t>
-        </is>
-      </c>
-      <c r="I125" s="0" t="inlineStr">
-        <is>
-          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="137">
       <c r="A126" s="202" t="inlineStr">
         <is>
+          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
+        </is>
+      </c>
+      <c r="B126" s="202" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C126" s="203" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D126" s="202" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
+      <c r="I126" s="0" t="inlineStr">
+        <is>
+          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="14.25" customHeight="1" s="137">
+      <c r="A127" s="202" t="inlineStr">
+        <is>
+          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
+        </is>
+      </c>
+      <c r="B127" s="202" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C127" s="203" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D127" s="202" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
+      <c r="I127" s="0" t="inlineStr">
+        <is>
+          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="14.25" customHeight="1" s="137">
+      <c r="A128" s="202" t="inlineStr">
+        <is>
           <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs (3 of 3)</t>
         </is>
       </c>
-      <c r="B126" s="202" t="inlineStr">
+      <c r="B128" s="202" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C126" s="203" t="n">
+      <c r="C128" s="203" t="n">
         <v>7581</v>
       </c>
-      <c r="D126" s="202" t="inlineStr">
+      <c r="D128" s="202" t="inlineStr">
         <is>
           <t>2025-12-24</t>
         </is>
       </c>
-      <c r="I126" s="0" t="inlineStr">
+      <c r="I128" s="0" t="inlineStr">
         <is>
           <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="14.25" customHeight="1" s="137">
-      <c r="A127" s="0" t="inlineStr">
+    <row r="129" ht="14.25" customHeight="1" s="137">
+      <c r="A129" s="0" t="inlineStr">
         <is>
           <t>Newstar 2025 total</t>
         </is>
       </c>
-      <c r="C127" s="203">
-        <f>SUM(C123:C125)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="128" ht="14.25" customHeight="1" s="137"/>
-    <row r="129" ht="14.25" customHeight="1" s="137">
-      <c r="A129" s="201" t="inlineStr">
-        <is>
-          <t>2025 Mercury Fortuna inventory — Venus + Roman Gold Belt LOCKED; Aug $20k unnamed ASK</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="14.25" customHeight="1" s="137">
-      <c r="A130" s="181" t="inlineStr">
-        <is>
-          <t>Bronze head of a goddess, likely Venus — Fortuna inventory</t>
-        </is>
-      </c>
-      <c r="B130" s="181" t="inlineStr">
+      <c r="C129" s="183">
+        <f>SUM(C126:C128)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130" ht="14.25" customHeight="1" s="137"/>
+    <row r="131" ht="14.25" customHeight="1" s="137">
+      <c r="A131" s="236" t="inlineStr">
+        <is>
+          <t>2025 Mercury Fortuna — Venus + Belt SOLD 2025 (see Sales 2025 rows 78–79); Aug $20k unnamed still ASK</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="14.25" customHeight="1" s="137">
+      <c r="A132" s="181" t="inlineStr">
+        <is>
+          <t>SOLD 2025 — Venus joint (see Sales 2025 row 79). Not unsold inventory.</t>
+        </is>
+      </c>
+      <c r="B132" s="181" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C130" s="203" t="n">
+      <c r="C132" s="183" t="n"/>
+      <c r="D132" s="202" t="inlineStr">
+        <is>
+          <t>2025-05-09</t>
+        </is>
+      </c>
+      <c r="I132" s="208" t="inlineStr">
+        <is>
+          <t>Moved to sold lots. EPGC proceeds $26,000 / Cost $20,000 / net $6,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="14.25" customHeight="1" s="137">
+      <c r="A133" s="181" t="inlineStr">
+        <is>
+          <t>SOLD 2025 — Roman Gold Belt to L5 (see Sales 2025 row 78). Not unsold inventory.</t>
+        </is>
+      </c>
+      <c r="B133" s="181" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C133" s="183" t="n"/>
+      <c r="D133" s="202" t="inlineStr">
+        <is>
+          <t>2025-07-21</t>
+        </is>
+      </c>
+      <c r="I133" s="208" t="inlineStr">
+        <is>
+          <t>Moved to sold lots. L5 $50,000 / Cost $45,000 / net $5,000. Remaining L5 not attached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="14.25" customHeight="1" s="137">
+      <c r="A134" s="185" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere — object still unnamed (native 8/18 = Monarch 8/15)</t>
+        </is>
+      </c>
+      <c r="B134" s="185" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C134" s="139" t="n">
         <v>20000</v>
       </c>
-      <c r="D130" s="202" t="inlineStr">
-        <is>
-          <t>2025-05-09</t>
-        </is>
-      </c>
-      <c r="I130" s="208" t="inlineStr">
-        <is>
-          <t>LOCKED 2026-09-20 from Mercury native CSV note. Parked Cost. Not sold 2025 — not in sold-lot Cost. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="14.25" customHeight="1" s="137">
-      <c r="A131" s="181" t="inlineStr">
-        <is>
-          <t>Roman Gold Belt — Fortuna inventory</t>
-        </is>
-      </c>
-      <c r="B131" s="181" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C131" s="203" t="n">
-        <v>45000</v>
-      </c>
-      <c r="D131" s="202" t="inlineStr">
-        <is>
-          <t>2025-07-21</t>
-        </is>
-      </c>
-      <c r="I131" s="208" t="inlineStr">
-        <is>
-          <t>LOCKED 2026-09-20 from Mercury native CSV note. Parked Cost. Not sold 2025 — not in sold-lot Cost. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="14.25" customHeight="1" s="137">
-      <c r="A132" s="185" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere — object still unnamed (native 8/18 = Monarch 8/15)</t>
-        </is>
-      </c>
-      <c r="B132" s="185" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C132" s="157" t="n">
+      <c r="D134" s="185" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
+      <c r="E134" s="185" t="n"/>
+      <c r="F134" s="185" t="n"/>
+      <c r="G134" s="185" t="n"/>
+      <c r="H134" s="185" t="n"/>
+      <c r="I134" s="190" t="inlineStr">
+        <is>
+          <t>ASK: same $20,000 as Mercury native 2025-08-18. No object name. Not Venus. Not belt. Do not add to sold Cost. Not a second unique txn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="14.25" customHeight="1" s="137">
+      <c r="A135" s="237" t="inlineStr">
+        <is>
+          <t>Fortuna unnamed remaining 2025 (excl. seals $13,000 sold + Venus $20,000 sold + Belt $45,000 sold)</t>
+        </is>
+      </c>
+      <c r="C135" s="139" t="n">
         <v>20000</v>
       </c>
-      <c r="D132" s="200" t="inlineStr">
-        <is>
-          <t>2025-08-15</t>
-        </is>
-      </c>
-      <c r="I132" s="190" t="inlineStr">
-        <is>
-          <t>ASK: same $20,000 as Mercury native 2025-08-18. No object name. Do not add to sold Cost. Not a second unique txn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="14.25" customHeight="1" s="137">
-      <c r="A133" s="0" t="inlineStr">
-        <is>
-          <t>Fortuna unnamed remaining 2025 (excl. seals $13,000 + Venus $20,000 + Belt $45,000)</t>
-        </is>
-      </c>
-      <c r="C133" s="157" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="134" ht="14.25" customHeight="1" s="137"/>
-    <row r="135" ht="14.25" customHeight="1" s="137"/>
+    </row>
     <row r="136" ht="14.25" customHeight="1" s="137"/>
     <row r="137" ht="14.25" customHeight="1" s="137"/>
     <row r="138" ht="14.25" customHeight="1" s="137"/>
@@ -32066,10 +32316,9 @@
     <row r="999" ht="14.25" customHeight="1" s="137"/>
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A134:I134"/>
+  <mergeCells count="3">
     <mergeCell ref="A119:I119"/>
-    <mergeCell ref="A79:I79"/>
+    <mergeCell ref="A81:I81"/>
     <mergeCell ref="A122:I122"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -32497,7 +32746,7 @@
       <c r="B27" s="94" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="137">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>BOM PAYMEN $21,500 = Form 1099-NEC (personal, Jacob). NOT EPGC Consultant. JAKE C / SEFOF reimbursements excluded. Not tax advice.</t>
         </is>

</xml_diff>

<commit_message>
Lock August Fortuna joint sale and per-invoice EOEB classifier.
August Fortuna is a second Erdal joint (Cost $20,000 / proceeds $25,000, net $5,000) on EPGC Art Sales October. EOEB remainder $130,270 stays UNALLOCATED per invoice (proposed FEE, not dumped). Income I8 is $39,055.06.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
+++ b/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
@@ -30,6 +30,7 @@
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="169" formatCode="_([$CAD]\ * #,##0.00_);_([$CAD]\ * \(#,##0.00\);_([$CAD]\ * &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="37">
     <font>
@@ -1709,7 +1710,7 @@
         <v>20000</v>
       </c>
       <c r="I8" s="183" t="n">
-        <v>34055.06</v>
+        <v>39055.06</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="137">
@@ -1785,7 +1786,7 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="182" t="inlineStr">
         <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $34,055.06 = prior MATCHED nets $23,055.06 (Berk lots + seals $1,000 + mosaics $15,000) + Belt net $5,000 + Venus EPGC-share net $6,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 / other L5 $37,396.32 / other Erdal IN $31,000 / Aysel $50,000 / Fortuna Aug $20,000 still ASK. Not tax advice.</t>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $39,055.06 = prior MATCHED nets $23,055.06 (Berk lots + seals $1,000 + mosaics $15,000) + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 stays UNALLOCATED (per-invoice Deal Classifier; proposed FEE, no matching Cost — not dumped). Other L5 $37,396.32 / Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -8896,12 +8897,12 @@
       </c>
       <c r="C11" s="226" t="inlineStr">
         <is>
-          <t>34,055.06</t>
+          <t>39,055.06</t>
         </is>
       </c>
       <c r="D11" s="226" t="inlineStr">
         <is>
-          <t>Prior MATCHED $23,055.06 + Belt net $5,000 + Venus EPGC-share net $6,000. Sale 6428 and Aquinas wait on Cost.</t>
+          <t>Prior MATCHED $23,055.06 + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Sale 6428 and Aquinas wait on Cost.</t>
         </is>
       </c>
       <c r="E11" s="226" t="inlineStr">
@@ -9247,12 +9248,12 @@
       </c>
       <c r="C24" s="226" t="inlineStr">
         <is>
-          <t>14,000 Jan + 136,000 Feb + 76,000 July = 226,000</t>
+          <t>14,000 Jan + 136,000 Feb + 76,000 July + 25,000 Oct = 251,000</t>
         </is>
       </c>
       <c r="D24" s="226" t="inlineStr">
         <is>
-          <t>Gross sale cash. July = Belt L5 $50,000 + Venus remittance $26,000. Do not dump EOEB $130,270 or other L5 $37,396.32.</t>
+          <t>Gross sale cash. July = Belt L5 $50,000 + Venus $26,000. October = August Fortuna joint remittance $25,000. Do not dump EOEB $130,270 or other L5 $37,396.32.</t>
         </is>
       </c>
       <c r="E24" s="226" t="inlineStr">
@@ -9323,17 +9324,17 @@
       </c>
       <c r="B27" s="224" t="inlineStr">
         <is>
-          <t>Seals / lots / mosaics / Belt / Venus</t>
+          <t>Seals / lots / mosaics / Belt / Venus / August joint</t>
         </is>
       </c>
       <c r="C27" s="224" t="inlineStr">
         <is>
-          <t>rows 70–79</t>
+          <t>rows 70–80</t>
         </is>
       </c>
       <c r="D27" s="224" t="inlineStr">
         <is>
-          <t>2022–2024 lots stay. 2025 adds Roman Gold Belt SALE and Venus joint SALE (EPGC share).</t>
+          <t>2022–2024 lots stay. 2025 adds Belt SALE, Venus joint SALE, August Fortuna joint SALE.</t>
         </is>
       </c>
       <c r="E27" s="226" t="inlineStr">
@@ -9464,7 +9465,7 @@
       </c>
       <c r="B34" s="224" t="inlineStr">
         <is>
-          <t>Mixed art + consultant. Invoice split still ASK. Belt $50k is locked SALE; remaining L5 is not.</t>
+          <t>EOEB remainder is per-invoice UNALLOCATED (proposed FEE, no matching Cost). Not dumped. Belt $50k SALE; remaining L5 not attached.</t>
         </is>
       </c>
       <c r="C34" s="224" t="inlineStr"/>
@@ -9620,7 +9621,7 @@
     <row r="43">
       <c r="A43" s="229" t="inlineStr">
         <is>
-          <t>EPGC Art Sales vs $226,000</t>
+          <t>EPGC Art Sales vs $251,000</t>
         </is>
       </c>
       <c r="B43" s="230">
@@ -9628,7 +9629,7 @@
         <v/>
       </c>
       <c r="C43" s="230" t="n">
-        <v>226000</v>
+        <v>251000</v>
       </c>
       <c r="D43" s="229">
         <f>IF(ROUND(B43,2)=ROUND(C43,2),"MATCH","FAIL")</f>
@@ -9669,6 +9670,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="238" t="inlineStr">
         <is>
@@ -9699,7 +9701,7 @@
       </c>
       <c r="E49" s="238" t="inlineStr"/>
     </row>
-    <row r="50" ht="32" customHeight="1" s="137">
+    <row r="50" ht="36" customHeight="1" s="137">
       <c r="A50" s="208" t="inlineStr">
         <is>
           <t>SALE</t>
@@ -9715,9 +9717,13 @@
           <t>Roman Gold Belt L5 $50,000 / Cost $45,000</t>
         </is>
       </c>
-      <c r="D50" s="208" t="inlineStr"/>
-    </row>
-    <row r="51" ht="32" customHeight="1" s="137">
+      <c r="D50" s="208" t="inlineStr">
+        <is>
+          <t>Remaining L5 $37,396.32</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="36" customHeight="1" s="137">
       <c r="A51" s="208" t="inlineStr">
         <is>
           <t>SALE (joint, EPGC share)</t>
@@ -9730,12 +9736,16 @@
       </c>
       <c r="C51" s="208" t="inlineStr">
         <is>
-          <t>Venus Erdal remittance $26,000 / EPGC Cost $20,000</t>
-        </is>
-      </c>
-      <c r="D51" s="208" t="inlineStr"/>
-    </row>
-    <row r="52" ht="32" customHeight="1" s="137">
+          <t>Venus $26,000 / Cost $20,000; August unnamed $25,000 / Cost $20,000</t>
+        </is>
+      </c>
+      <c r="D51" s="208" t="inlineStr">
+        <is>
+          <t>11/7 $6,000 FORTUNA PAYMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1" s="137">
       <c r="A52" s="208" t="inlineStr">
         <is>
           <t>FEE</t>
@@ -9751,9 +9761,13 @@
           <t>David Aaron June $13,595 Consultant; Wise write-ups $992.80 Fees</t>
         </is>
       </c>
-      <c r="D52" s="208" t="inlineStr"/>
-    </row>
-    <row r="53" ht="32" customHeight="1" s="137">
+      <c r="D52" s="208" t="inlineStr">
+        <is>
+          <t>EOEB remainder proposed FEE but not locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="36" customHeight="1" s="137">
       <c r="A53" s="208" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -9771,23 +9785,27 @@
       </c>
       <c r="D53" s="208" t="inlineStr"/>
     </row>
-    <row r="54" ht="32" customHeight="1" s="137">
+    <row r="54" ht="36" customHeight="1" s="137">
       <c r="A54" s="190" t="inlineStr">
         <is>
-          <t>INVENTORY</t>
+          <t>UNALLOCATED</t>
         </is>
       </c>
       <c r="B54" s="190" t="inlineStr">
         <is>
-          <t>Named or unnamed purchase still unsold</t>
+          <t>Show the invoice; do not dump onto Consultant or Art Sales</t>
         </is>
       </c>
       <c r="C54" s="190" t="inlineStr">
         <is>
-          <t>Fortuna Aug unnamed $20,000</t>
-        </is>
-      </c>
-      <c r="D54" s="190" t="inlineStr"/>
+          <t>EOEB remainder $130,270.00 per-invoice (see DEAL_CLASSIFIER.csv)</t>
+        </is>
+      </c>
+      <c r="D54" s="190" t="inlineStr">
+        <is>
+          <t>L5 remainder $37,396.32; Aysel $50,000</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="32" customHeight="1" s="137">
       <c r="A55" s="190" t="inlineStr">
@@ -23410,8 +23428,8 @@
       <c r="J53" s="179" t="n">
         <v>0</v>
       </c>
-      <c r="K53" s="179" t="n">
-        <v>0</v>
+      <c r="K53" s="183" t="n">
+        <v>25000</v>
       </c>
       <c r="L53" s="179" t="n">
         <v>0</v>
@@ -24200,10 +24218,10 @@
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="137"/>
-    <row r="75" ht="72" customHeight="1" s="137">
+    <row r="75" ht="84" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) = $226,000. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 and other L5 $37,396.32 MIXED PATTERN CONFIRMED — invoice-level split still ASK; not dumped. Other Erdal IN 10/9 $25,000 and 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Fortuna Aug unnamed $20,000 still ASK (not Venus, not belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD — cash on Art Sales, not in I8. Venus Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $251,000. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE, no matching dealer Cost; Fortuna joints are NOT EOEB Cost) — not dumped onto Consultant or Art Sales. Other L5 $37,396.32 MIXED — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD — cash on Art Sales, not in I8. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -27752,7 +27770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z135"/>
+  <dimension ref="A1:Z136"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="47.86" customWidth="1" style="137" min="1" max="1"/>
@@ -30572,88 +30590,113 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="14.25" customHeight="1" s="137">
-      <c r="A80" s="184" t="inlineStr">
+    <row r="80" ht="64" customHeight="1" s="137">
+      <c r="A80" s="181" t="inlineStr">
+        <is>
+          <t>August Fortuna joint — unnamed object (EPGC share)</t>
+        </is>
+      </c>
+      <c r="B80" s="181" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere</t>
+        </is>
+      </c>
+      <c r="C80" s="183" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D80" s="209" t="n">
+        <v>45884</v>
+      </c>
+      <c r="E80" s="181" t="inlineStr">
+        <is>
+          <t>Erdal Dere</t>
+        </is>
+      </c>
+      <c r="F80" s="183" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G80" s="209" t="n">
+        <v>45939</v>
+      </c>
+      <c r="H80" s="183">
+        <f>F80-C80</f>
+        <v/>
+      </c>
+      <c r="I80" s="208" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 joint SALE (EPGC share). Another joint investment with Erdal (user 2026-09-21). He sold; Jacob got capital + earnings. EPGC Cost: Fortuna 8/15 −$20,000 (Mercury native 8/18, same cash; object unnamed). Working remittance: Erdal Dere IN 10/9 +$25,000 = $20,000 capital + $5,000 earnings. Sale Price on this register is EPGC proceeds ($25,000), not the object’s full hammer. Hits EPGC Art Sales October. 7/24 is Venus, not August. 11/7 $6,000 FORTUNA PAYMENT still ASK. Classifier: SALE (joint, EPGC share). Not consultant. Not unsold inventory. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="J80" s="181" t="n"/>
+      <c r="K80" s="181" t="inlineStr">
+        <is>
+          <t>SALE (joint, EPGC share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="64" customHeight="1" s="137">
+      <c r="A81" s="184" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H80" s="235">
-        <f>SUM(H51:H75)+H78+H79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" ht="64" customHeight="1" s="137">
-      <c r="A81" s="208" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000 (Sale Price = remittance, not full hammer). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 or other L5 $37,396.32. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="14.25" customHeight="1" s="137">
-      <c r="A82" s="119" t="inlineStr">
+      <c r="H81" s="235">
+        <f>SUM(H51:H75)+H78+H79+H80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" ht="72" customHeight="1" s="137">
+      <c r="A82" s="208" t="inlineStr">
+        <is>
+          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 (see Deal Classifier per invoice) or other L5 $37,396.32. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="14.25" customHeight="1" s="137">
+      <c r="A83" s="119" t="inlineStr">
         <is>
           <t>Art Purchases/Inventory</t>
         </is>
       </c>
-      <c r="B82" s="120" t="n"/>
-      <c r="C82" s="100" t="n"/>
-      <c r="D82" s="101" t="n"/>
-      <c r="E82" s="99" t="n"/>
-      <c r="F82" s="100" t="n"/>
-      <c r="G82" s="101" t="n"/>
-      <c r="H82" s="99" t="n"/>
-      <c r="I82" s="121" t="n"/>
-      <c r="J82" s="99" t="n"/>
-      <c r="K82" s="99" t="n"/>
-      <c r="L82" s="99" t="n"/>
-      <c r="M82" s="99" t="n"/>
-      <c r="N82" s="99" t="n"/>
-      <c r="O82" s="99" t="n"/>
-      <c r="P82" s="99" t="n"/>
-      <c r="Q82" s="99" t="n"/>
-      <c r="R82" s="99" t="n"/>
-      <c r="S82" s="99" t="n"/>
-      <c r="T82" s="99" t="n"/>
-      <c r="U82" s="99" t="n"/>
-      <c r="V82" s="99" t="n"/>
-      <c r="W82" s="99" t="n"/>
-      <c r="X82" s="99" t="n"/>
-      <c r="Y82" s="99" t="n"/>
-      <c r="Z82" s="99" t="n"/>
-    </row>
-    <row r="83" ht="14.25" customHeight="1" s="137">
-      <c r="A83" s="122" t="inlineStr">
-        <is>
-          <t>30 Paleothic and Neolithic Stone Tools</t>
-        </is>
-      </c>
-      <c r="B83" s="116" t="inlineStr">
-        <is>
-          <t>Holestein</t>
-        </is>
-      </c>
-      <c r="C83" s="88" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E83" s="105" t="n"/>
+      <c r="B83" s="120" t="n"/>
+      <c r="C83" s="100" t="n"/>
+      <c r="D83" s="101" t="n"/>
+      <c r="E83" s="99" t="n"/>
+      <c r="F83" s="100" t="n"/>
+      <c r="G83" s="101" t="n"/>
+      <c r="H83" s="99" t="n"/>
+      <c r="I83" s="121" t="n"/>
+      <c r="J83" s="99" t="n"/>
+      <c r="K83" s="99" t="n"/>
+      <c r="L83" s="99" t="n"/>
+      <c r="M83" s="99" t="n"/>
+      <c r="N83" s="99" t="n"/>
+      <c r="O83" s="99" t="n"/>
+      <c r="P83" s="99" t="n"/>
+      <c r="Q83" s="99" t="n"/>
+      <c r="R83" s="99" t="n"/>
+      <c r="S83" s="99" t="n"/>
+      <c r="T83" s="99" t="n"/>
+      <c r="U83" s="99" t="n"/>
+      <c r="V83" s="99" t="n"/>
+      <c r="W83" s="99" t="n"/>
+      <c r="X83" s="99" t="n"/>
+      <c r="Y83" s="99" t="n"/>
+      <c r="Z83" s="99" t="n"/>
     </row>
     <row r="84" ht="14.25" customHeight="1" s="137">
       <c r="A84" s="122" t="inlineStr">
         <is>
-          <t>A Tairona Figure</t>
+          <t>30 Paleothic and Neolithic Stone Tools</t>
         </is>
       </c>
       <c r="B84" s="116" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Holestein</t>
         </is>
       </c>
       <c r="C84" s="88" t="n">
-        <v>250</v>
-      </c>
-      <c r="D84" s="92" t="n">
-        <v>45119</v>
+        <v>4000</v>
       </c>
       <c r="E84" s="105" t="n"/>
     </row>
@@ -30669,7 +30712,7 @@
         </is>
       </c>
       <c r="C85" s="88" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D85" s="92" t="n">
         <v>45119</v>
@@ -30679,26 +30722,26 @@
     <row r="86" ht="14.25" customHeight="1" s="137">
       <c r="A86" s="122" t="inlineStr">
         <is>
-          <t>A Pair of Greek Bronze Greeves</t>
+          <t>A Tairona Figure</t>
         </is>
       </c>
       <c r="B86" s="116" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C86" s="88" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D86" s="92" t="n">
-        <v>45145</v>
+        <v>45119</v>
       </c>
       <c r="E86" s="105" t="n"/>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="137">
       <c r="A87" s="122" t="inlineStr">
         <is>
-          <t>An Illyrian Bronze Helmet</t>
+          <t>A Pair of Greek Bronze Greeves</t>
         </is>
       </c>
       <c r="B87" s="116" t="inlineStr">
@@ -30707,58 +30750,57 @@
         </is>
       </c>
       <c r="C87" s="88" t="n">
-        <v>551.25</v>
+        <v>200</v>
       </c>
       <c r="D87" s="92" t="n">
-        <v>45114</v>
+        <v>45145</v>
       </c>
       <c r="E87" s="105" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="137">
       <c r="A88" s="122" t="inlineStr">
         <is>
-          <t>An Egyptian Faience Ibis</t>
-        </is>
-      </c>
-      <c r="B88" s="104" t="inlineStr">
-        <is>
-          <t>Hindman</t>
+          <t>An Illyrian Bronze Helmet</t>
+        </is>
+      </c>
+      <c r="B88" s="116" t="inlineStr">
+        <is>
+          <t>ebay</t>
         </is>
       </c>
       <c r="C88" s="88" t="n">
-        <v>375</v>
+        <v>551.25</v>
       </c>
       <c r="D88" s="92" t="n">
-        <v>44343</v>
-      </c>
-      <c r="E88" s="92" t="n"/>
-      <c r="F88" s="88" t="n"/>
-      <c r="I88" s="105" t="n"/>
+        <v>45114</v>
+      </c>
+      <c r="E88" s="105" t="n"/>
     </row>
     <row r="89" ht="14.25" customHeight="1" s="137">
       <c r="A89" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
+          <t>An Egyptian Faience Ibis</t>
         </is>
       </c>
       <c r="B89" s="104" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C89" s="88" t="n">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="D89" s="92" t="n">
-        <v>44548</v>
-      </c>
+        <v>44343</v>
+      </c>
+      <c r="E89" s="92" t="n"/>
       <c r="F89" s="88" t="n"/>
       <c r="I89" s="105" t="n"/>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="137">
       <c r="A90" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
         </is>
       </c>
       <c r="B90" s="104" t="inlineStr">
@@ -30778,7 +30820,7 @@
     <row r="91" ht="14.25" customHeight="1" s="137">
       <c r="A91" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
         </is>
       </c>
       <c r="B91" s="104" t="inlineStr">
@@ -30798,19 +30840,19 @@
     <row r="92" ht="14.25" customHeight="1" s="137">
       <c r="A92" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
         </is>
       </c>
       <c r="B92" s="104" t="inlineStr">
         <is>
-          <t>Pace African Art</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C92" s="88" t="n">
-        <v>1000</v>
+        <v>293</v>
       </c>
       <c r="D92" s="92" t="n">
-        <v>44562</v>
+        <v>44548</v>
       </c>
       <c r="F92" s="88" t="n"/>
       <c r="I92" s="105" t="n"/>
@@ -30818,16 +30860,19 @@
     <row r="93" ht="14.25" customHeight="1" s="137">
       <c r="A93" s="122" t="inlineStr">
         <is>
-          <t>Carved Ostrish Egg</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B93" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etsy </t>
+          <t>Pace African Art</t>
         </is>
       </c>
       <c r="C93" s="88" t="n">
-        <v>90</v>
+        <v>1000</v>
+      </c>
+      <c r="D93" s="92" t="n">
+        <v>44562</v>
       </c>
       <c r="F93" s="88" t="n"/>
       <c r="I93" s="105" t="n"/>
@@ -30835,16 +30880,16 @@
     <row r="94" ht="14.25" customHeight="1" s="137">
       <c r="A94" s="122" t="inlineStr">
         <is>
-          <t>Carved Goose Egg</t>
+          <t>Carved Ostrish Egg</t>
         </is>
       </c>
       <c r="B94" s="104" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t xml:space="preserve">Etsy </t>
         </is>
       </c>
       <c r="C94" s="88" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="F94" s="88" t="n"/>
       <c r="I94" s="105" t="n"/>
@@ -30861,7 +30906,7 @@
         </is>
       </c>
       <c r="C95" s="88" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F95" s="88" t="n"/>
       <c r="I95" s="105" t="n"/>
@@ -30869,31 +30914,29 @@
     <row r="96" ht="14.25" customHeight="1" s="137">
       <c r="A96" s="122" t="inlineStr">
         <is>
-          <t>Quimbaya Figure (Gift)</t>
+          <t>Carved Goose Egg</t>
         </is>
       </c>
       <c r="B96" s="104" t="inlineStr">
         <is>
-          <t>Jeffrey Norris</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C96" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="D96" s="92" t="n">
-        <v>45079</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F96" s="88" t="n"/>
       <c r="I96" s="105" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1" s="137">
       <c r="A97" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal (Gift)</t>
+          <t>Quimbaya Figure (Gift)</t>
         </is>
       </c>
       <c r="B97" s="104" t="inlineStr">
         <is>
-          <t>Aquinas Hobor</t>
+          <t>Jeffrey Norris</t>
         </is>
       </c>
       <c r="C97" s="88" t="n">
@@ -30907,7 +30950,7 @@
     <row r="98" ht="14.25" customHeight="1" s="137">
       <c r="A98" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>A Saharan Stone Discoidal (Gift)</t>
         </is>
       </c>
       <c r="B98" s="104" t="inlineStr">
@@ -30915,31 +30958,30 @@
           <t>Aquinas Hobor</t>
         </is>
       </c>
-      <c r="C98" s="103" t="n">
-        <v>500</v>
+      <c r="C98" s="88" t="n">
+        <v>10</v>
       </c>
       <c r="D98" s="92" t="n">
         <v>45079</v>
       </c>
-      <c r="F98" s="88" t="n"/>
       <c r="I98" s="105" t="n"/>
     </row>
     <row r="99" ht="14.25" customHeight="1" s="137">
       <c r="A99" s="122" t="inlineStr">
         <is>
-          <t>Two Songye and Bozo Vessels</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B99" s="104" t="inlineStr">
         <is>
-          <t>Hindman</t>
+          <t>Aquinas Hobor</t>
         </is>
       </c>
       <c r="C99" s="103" t="n">
-        <v>138.91</v>
+        <v>500</v>
       </c>
       <c r="D99" s="92" t="n">
-        <v>45211</v>
+        <v>45079</v>
       </c>
       <c r="F99" s="88" t="n"/>
       <c r="I99" s="105" t="n"/>
@@ -30947,19 +30989,19 @@
     <row r="100" ht="14.25" customHeight="1" s="137">
       <c r="A100" s="122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sword 9th Century </t>
+          <t>Two Songye and Bozo Vessels</t>
         </is>
       </c>
       <c r="B100" s="104" t="inlineStr">
         <is>
-          <t>Zevantiques</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C100" s="103" t="n">
-        <v>3000</v>
+        <v>138.91</v>
       </c>
       <c r="D100" s="92" t="n">
-        <v>45311</v>
+        <v>45211</v>
       </c>
       <c r="F100" s="88" t="n"/>
       <c r="I100" s="105" t="n"/>
@@ -30967,19 +31009,19 @@
     <row r="101" ht="14.25" customHeight="1" s="137">
       <c r="A101" s="122" t="inlineStr">
         <is>
-          <t>A Roman Marble Plaque with Insciption</t>
+          <t xml:space="preserve">Sword 9th Century </t>
         </is>
       </c>
       <c r="B101" s="104" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Zevantiques</t>
         </is>
       </c>
       <c r="C101" s="103" t="n">
-        <v>1331.41</v>
+        <v>3000</v>
       </c>
       <c r="D101" s="92" t="n">
-        <v>45546</v>
+        <v>45311</v>
       </c>
       <c r="F101" s="88" t="n"/>
       <c r="I101" s="105" t="n"/>
@@ -30987,7 +31029,7 @@
     <row r="102" ht="14.25" customHeight="1" s="137">
       <c r="A102" s="122" t="inlineStr">
         <is>
-          <t>Erotic Intaglio Finger Ring</t>
+          <t>A Roman Marble Plaque with Insciption</t>
         </is>
       </c>
       <c r="B102" s="104" t="inlineStr">
@@ -30996,85 +31038,94 @@
         </is>
       </c>
       <c r="C102" s="103" t="n">
-        <v>205.07</v>
+        <v>1331.41</v>
       </c>
       <c r="D102" s="92" t="n">
-        <v>45446</v>
+        <v>45546</v>
       </c>
       <c r="F102" s="88" t="n"/>
       <c r="I102" s="105" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="137">
-      <c r="B103" s="104" t="n"/>
-      <c r="C103" s="103" t="n"/>
-      <c r="D103" s="92" t="n"/>
+      <c r="A103" s="122" t="inlineStr">
+        <is>
+          <t>Erotic Intaglio Finger Ring</t>
+        </is>
+      </c>
+      <c r="B103" s="104" t="inlineStr">
+        <is>
+          <t>ebay</t>
+        </is>
+      </c>
+      <c r="C103" s="103" t="n">
+        <v>205.07</v>
+      </c>
+      <c r="D103" s="92" t="n">
+        <v>45446</v>
+      </c>
       <c r="F103" s="88" t="n"/>
       <c r="I103" s="105" t="n"/>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="137">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
       <c r="B104" s="104" t="n"/>
-      <c r="C104" s="86" t="n"/>
+      <c r="C104" s="103" t="n"/>
+      <c r="D104" s="92" t="n"/>
       <c r="F104" s="88" t="n"/>
       <c r="I104" s="105" t="n"/>
     </row>
     <row r="105" ht="14.25" customHeight="1" s="137">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
       <c r="B105" s="104" t="n"/>
-      <c r="C105" s="88" t="n"/>
+      <c r="C105" s="86" t="n"/>
       <c r="F105" s="88" t="n"/>
       <c r="I105" s="105" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="137">
-      <c r="A106" s="119" t="inlineStr">
+      <c r="B106" s="104" t="n"/>
+      <c r="C106" s="88" t="n"/>
+      <c r="F106" s="88" t="n"/>
+      <c r="I106" s="105" t="n"/>
+    </row>
+    <row r="107" ht="14.25" customHeight="1" s="137">
+      <c r="A107" s="119" t="inlineStr">
         <is>
           <t>Office/Business Inventory</t>
         </is>
       </c>
-      <c r="B106" s="120" t="n"/>
-      <c r="C106" s="100" t="n"/>
-      <c r="D106" s="99" t="n"/>
-      <c r="E106" s="99" t="n"/>
-      <c r="F106" s="100" t="n"/>
-      <c r="G106" s="99" t="n"/>
-      <c r="H106" s="99" t="n"/>
-      <c r="I106" s="121" t="n"/>
-      <c r="J106" s="99" t="n"/>
-      <c r="K106" s="99" t="n"/>
-      <c r="L106" s="99" t="n"/>
-      <c r="M106" s="99" t="n"/>
-      <c r="N106" s="99" t="n"/>
-      <c r="O106" s="99" t="n"/>
-      <c r="P106" s="99" t="n"/>
-      <c r="Q106" s="99" t="n"/>
-      <c r="R106" s="99" t="n"/>
-      <c r="S106" s="99" t="n"/>
-      <c r="T106" s="99" t="n"/>
-      <c r="U106" s="99" t="n"/>
-      <c r="V106" s="99" t="n"/>
-      <c r="W106" s="99" t="n"/>
-      <c r="X106" s="99" t="n"/>
-      <c r="Y106" s="99" t="n"/>
-      <c r="Z106" s="99" t="n"/>
-    </row>
-    <row r="107" ht="14.25" customHeight="1" s="137">
-      <c r="A107" s="122" t="inlineStr">
-        <is>
-          <t>Sofa</t>
-        </is>
-      </c>
-      <c r="B107" s="104" t="n"/>
-      <c r="C107" s="88" t="n"/>
-      <c r="F107" s="88" t="n"/>
-      <c r="I107" s="105" t="n"/>
+      <c r="B107" s="120" t="n"/>
+      <c r="C107" s="100" t="n"/>
+      <c r="D107" s="99" t="n"/>
+      <c r="E107" s="99" t="n"/>
+      <c r="F107" s="100" t="n"/>
+      <c r="G107" s="99" t="n"/>
+      <c r="H107" s="99" t="n"/>
+      <c r="I107" s="121" t="n"/>
+      <c r="J107" s="99" t="n"/>
+      <c r="K107" s="99" t="n"/>
+      <c r="L107" s="99" t="n"/>
+      <c r="M107" s="99" t="n"/>
+      <c r="N107" s="99" t="n"/>
+      <c r="O107" s="99" t="n"/>
+      <c r="P107" s="99" t="n"/>
+      <c r="Q107" s="99" t="n"/>
+      <c r="R107" s="99" t="n"/>
+      <c r="S107" s="99" t="n"/>
+      <c r="T107" s="99" t="n"/>
+      <c r="U107" s="99" t="n"/>
+      <c r="V107" s="99" t="n"/>
+      <c r="W107" s="99" t="n"/>
+      <c r="X107" s="99" t="n"/>
+      <c r="Y107" s="99" t="n"/>
+      <c r="Z107" s="99" t="n"/>
     </row>
     <row r="108" ht="14.25" customHeight="1" s="137">
       <c r="A108" s="122" t="inlineStr">
         <is>
-          <t>Space Heater</t>
+          <t>Sofa</t>
         </is>
       </c>
       <c r="B108" s="104" t="n"/>
@@ -31085,7 +31136,7 @@
     <row r="109" ht="14.25" customHeight="1" s="137">
       <c r="A109" s="122" t="inlineStr">
         <is>
-          <t>Shelving</t>
+          <t>Space Heater</t>
         </is>
       </c>
       <c r="B109" s="104" t="n"/>
@@ -31096,7 +31147,7 @@
     <row r="110" ht="14.25" customHeight="1" s="137">
       <c r="A110" s="122" t="inlineStr">
         <is>
-          <t>Storage Bins</t>
+          <t>Shelving</t>
         </is>
       </c>
       <c r="B110" s="104" t="n"/>
@@ -31107,7 +31158,7 @@
     <row r="111" ht="14.25" customHeight="1" s="137">
       <c r="A111" s="122" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Storage Bins</t>
         </is>
       </c>
       <c r="B111" s="104" t="n"/>
@@ -31118,7 +31169,7 @@
     <row r="112" ht="14.25" customHeight="1" s="137">
       <c r="A112" s="122" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="B112" s="104" t="n"/>
@@ -31129,7 +31180,7 @@
     <row r="113" ht="14.25" customHeight="1" s="137">
       <c r="A113" s="122" t="inlineStr">
         <is>
-          <t>Art Library</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B113" s="104" t="n"/>
@@ -31140,7 +31191,7 @@
     <row r="114" ht="14.25" customHeight="1" s="137">
       <c r="A114" s="122" t="inlineStr">
         <is>
-          <t>Standing Desk</t>
+          <t>Art Library</t>
         </is>
       </c>
       <c r="B114" s="104" t="n"/>
@@ -31149,46 +31200,37 @@
       <c r="I114" s="105" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="137">
+      <c r="A115" s="122" t="inlineStr">
+        <is>
+          <t>Standing Desk</t>
+        </is>
+      </c>
       <c r="B115" s="104" t="n"/>
       <c r="C115" s="88" t="n"/>
       <c r="F115" s="88" t="n"/>
       <c r="I115" s="105" t="n"/>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="137">
-      <c r="A116" s="156" t="inlineStr">
-        <is>
-          <t>2025 CC inventory (not in Cost total until object is named)</t>
-        </is>
-      </c>
       <c r="B116" s="104" t="n"/>
       <c r="C116" s="88" t="n"/>
       <c r="F116" s="88" t="n"/>
       <c r="I116" s="105" t="n"/>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="137">
-      <c r="A117" s="0" t="inlineStr">
-        <is>
-          <t>Los Angeles Modern Auctions (inventory purchase)</t>
-        </is>
-      </c>
-      <c r="B117" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C117" s="157" t="n">
-        <v>6821.06</v>
-      </c>
-      <c r="D117" s="0" t="inlineStr">
-        <is>
-          <t>2025-07-24</t>
-        </is>
-      </c>
+      <c r="A117" s="156" t="inlineStr">
+        <is>
+          <t>2025 CC inventory (not in Cost total until object is named)</t>
+        </is>
+      </c>
+      <c r="B117" s="104" t="n"/>
+      <c r="C117" s="88" t="n"/>
+      <c r="F117" s="88" t="n"/>
+      <c r="I117" s="105" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1" s="137">
       <c r="A118" s="0" t="inlineStr">
         <is>
-          <t>Hindman LLC (inventory purchase)</t>
+          <t>Los Angeles Modern Auctions (inventory purchase)</t>
         </is>
       </c>
       <c r="B118" s="0" t="inlineStr">
@@ -31197,11 +31239,11 @@
         </is>
       </c>
       <c r="C118" s="157" t="n">
-        <v>282.24</v>
+        <v>6821.06</v>
       </c>
       <c r="D118" s="0" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>2025-07-24</t>
         </is>
       </c>
     </row>
@@ -31211,88 +31253,83 @@
           <t>Hindman LLC (inventory purchase)</t>
         </is>
       </c>
+      <c r="B119" s="0" t="inlineStr">
+        <is>
+          <t>Sapphire 5423</t>
+        </is>
+      </c>
+      <c r="C119" s="157" t="n">
+        <v>282.24</v>
+      </c>
+      <c r="D119" s="0" t="inlineStr">
+        <is>
+          <t>2025-04-03</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="14.25" customHeight="1" s="137">
       <c r="A120" s="0" t="inlineStr">
         <is>
+          <t>Hindman LLC (inventory purchase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="14.25" customHeight="1" s="137">
+      <c r="A121" s="0" t="inlineStr">
+        <is>
           <t>The Great Frame Up (inventory framing)</t>
         </is>
       </c>
-      <c r="B120" s="0" t="inlineStr">
+      <c r="B121" s="0" t="inlineStr">
         <is>
           <t>Sapphire 5423</t>
         </is>
       </c>
-      <c r="C120" s="157" t="n">
+      <c r="C121" s="157" t="n">
         <v>536.41</v>
       </c>
-      <c r="D120" s="0" t="inlineStr">
+      <c r="D121" s="0" t="inlineStr">
         <is>
           <t>2025-02-16</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="14.25" customHeight="1" s="137"/>
-    <row r="122" ht="14.25" customHeight="1" s="137">
-      <c r="A122" s="201" t="inlineStr">
+    <row r="122" ht="14.25" customHeight="1" s="137"/>
+    <row r="123" ht="14.25" customHeight="1" s="137">
+      <c r="A123" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury 8291 — David Aaron Limited is LOCKED consultant fee (not Art Sales)</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="14.25" customHeight="1" s="137">
-      <c r="A123" s="181" t="inlineStr">
+    <row r="124" ht="14.25" customHeight="1" s="137">
+      <c r="A124" s="181" t="inlineStr">
         <is>
           <t>NOT a 2025 art sale — David Aaron Limited consultant fee (EPGC Consultant June)</t>
         </is>
       </c>
-      <c r="B123" s="181" t="inlineStr">
+      <c r="B124" s="181" t="inlineStr">
         <is>
           <t>David Aaron Limited</t>
         </is>
       </c>
-      <c r="C123" s="181" t="n"/>
-      <c r="D123" s="181" t="n"/>
-      <c r="E123" s="181" t="n"/>
-      <c r="F123" s="183" t="n"/>
-      <c r="G123" s="206" t="n"/>
-      <c r="H123" s="206" t="n"/>
-      <c r="I123" s="181" t="inlineStr">
+      <c r="C124" s="181" t="n"/>
+      <c r="D124" s="181" t="n"/>
+      <c r="E124" s="181" t="n"/>
+      <c r="F124" s="183" t="n"/>
+      <c r="G124" s="206" t="n"/>
+      <c r="H124" s="206" t="n"/>
+      <c r="I124" s="181" t="inlineStr">
         <is>
           <t>LOCKED 2026-09-20: consultant fee, not a sale. $13,595 is on EPGC Consultant June. Not tax advice.</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="14.25" customHeight="1" s="137"/>
-    <row r="125" ht="14.25" customHeight="1" s="137">
-      <c r="A125" s="201" t="inlineStr">
+    <row r="125" ht="14.25" customHeight="1" s="137"/>
+    <row r="126" ht="14.25" customHeight="1" s="137">
+      <c r="A126" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury COGS — Newstar Jewelers (LOCKED jewelry fabrication)</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="14.25" customHeight="1" s="137">
-      <c r="A126" s="202" t="inlineStr">
-        <is>
-          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
-        </is>
-      </c>
-      <c r="B126" s="202" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C126" s="203" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D126" s="202" t="inlineStr">
-        <is>
-          <t>2025-10-14</t>
-        </is>
-      </c>
-      <c r="I126" s="0" t="inlineStr">
-        <is>
-          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
@@ -31312,7 +31349,7 @@
       </c>
       <c r="D127" s="202" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="I127" s="0" t="inlineStr">
@@ -31324,74 +31361,76 @@
     <row r="128" ht="14.25" customHeight="1" s="137">
       <c r="A128" s="202" t="inlineStr">
         <is>
+          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
+        </is>
+      </c>
+      <c r="B128" s="202" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C128" s="203" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D128" s="202" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
+      <c r="I128" s="0" t="inlineStr">
+        <is>
+          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="14.25" customHeight="1" s="137">
+      <c r="A129" s="202" t="inlineStr">
+        <is>
           <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs (3 of 3)</t>
         </is>
       </c>
-      <c r="B128" s="202" t="inlineStr">
+      <c r="B129" s="202" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C128" s="203" t="n">
+      <c r="C129" s="203" t="n">
         <v>7581</v>
       </c>
-      <c r="D128" s="202" t="inlineStr">
+      <c r="D129" s="202" t="inlineStr">
         <is>
           <t>2025-12-24</t>
         </is>
       </c>
-      <c r="I128" s="0" t="inlineStr">
+      <c r="I129" s="0" t="inlineStr">
         <is>
           <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="14.25" customHeight="1" s="137">
-      <c r="A129" s="0" t="inlineStr">
+    <row r="130" ht="14.25" customHeight="1" s="137">
+      <c r="A130" s="0" t="inlineStr">
         <is>
           <t>Newstar 2025 total</t>
         </is>
       </c>
-      <c r="C129" s="183">
-        <f>SUM(C126:C128)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="130" ht="14.25" customHeight="1" s="137"/>
-    <row r="131" ht="14.25" customHeight="1" s="137">
-      <c r="A131" s="236" t="inlineStr">
-        <is>
-          <t>2025 Mercury Fortuna — Venus + Belt SOLD 2025 (see Sales 2025 rows 78–79); Aug $20k unnamed still ASK</t>
-        </is>
-      </c>
-    </row>
+      <c r="C130" s="183">
+        <f>SUM(C127:C129)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131" ht="14.25" customHeight="1" s="137"/>
     <row r="132" ht="14.25" customHeight="1" s="137">
-      <c r="A132" s="181" t="inlineStr">
-        <is>
-          <t>SOLD 2025 — Venus joint (see Sales 2025 row 79). Not unsold inventory.</t>
-        </is>
-      </c>
-      <c r="B132" s="181" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C132" s="183" t="n"/>
-      <c r="D132" s="202" t="inlineStr">
-        <is>
-          <t>2025-05-09</t>
-        </is>
-      </c>
-      <c r="I132" s="208" t="inlineStr">
-        <is>
-          <t>Moved to sold lots. EPGC proceeds $26,000 / Cost $20,000 / net $6,000.</t>
+      <c r="A132" s="236" t="inlineStr">
+        <is>
+          <t>2025 Mercury Fortuna — Venus + Belt + August joint SOLD 2025 (see Sales 2025 rows 78–80); no unnamed Fortuna Cost left on 8291</t>
         </is>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="137">
       <c r="A133" s="181" t="inlineStr">
         <is>
-          <t>SOLD 2025 — Roman Gold Belt to L5 (see Sales 2025 row 78). Not unsold inventory.</t>
+          <t>SOLD 2025 — Venus joint (see Sales 2025 row 79). Not unsold inventory.</t>
         </is>
       </c>
       <c r="B133" s="181" t="inlineStr">
@@ -31402,55 +31441,75 @@
       <c r="C133" s="183" t="n"/>
       <c r="D133" s="202" t="inlineStr">
         <is>
+          <t>2025-05-09</t>
+        </is>
+      </c>
+      <c r="I133" s="208" t="inlineStr">
+        <is>
+          <t>Moved to sold lots. EPGC proceeds $26,000 / Cost $20,000 / net $6,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="14.25" customHeight="1" s="137">
+      <c r="A134" s="181" t="inlineStr">
+        <is>
+          <t>SOLD 2025 — Roman Gold Belt to L5 (see Sales 2025 row 78). Not unsold inventory.</t>
+        </is>
+      </c>
+      <c r="B134" s="181" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C134" s="183" t="n"/>
+      <c r="D134" s="202" t="inlineStr">
+        <is>
           <t>2025-07-21</t>
         </is>
       </c>
-      <c r="I133" s="208" t="inlineStr">
+      <c r="I134" s="208" t="inlineStr">
         <is>
           <t>Moved to sold lots. L5 $50,000 / Cost $45,000 / net $5,000. Remaining L5 not attached.</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="14.25" customHeight="1" s="137">
-      <c r="A134" s="185" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere — object still unnamed (native 8/18 = Monarch 8/15)</t>
-        </is>
-      </c>
-      <c r="B134" s="185" t="inlineStr">
+    <row r="135" ht="14.25" customHeight="1" s="137">
+      <c r="A135" s="181" t="inlineStr">
+        <is>
+          <t>SOLD 2025 — August Fortuna joint (see Sales 2025 row 80). Not unsold inventory.</t>
+        </is>
+      </c>
+      <c r="B135" s="185" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C134" s="139" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D134" s="185" t="inlineStr">
+      <c r="C135" s="183" t="n"/>
+      <c r="D135" s="185" t="inlineStr">
         <is>
           <t>2025-08-15</t>
         </is>
       </c>
-      <c r="E134" s="185" t="n"/>
-      <c r="F134" s="185" t="n"/>
-      <c r="G134" s="185" t="n"/>
-      <c r="H134" s="185" t="n"/>
-      <c r="I134" s="190" t="inlineStr">
-        <is>
-          <t>ASK: same $20,000 as Mercury native 2025-08-18. No object name. Not Venus. Not belt. Do not add to sold Cost. Not a second unique txn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="14.25" customHeight="1" s="137">
-      <c r="A135" s="237" t="inlineStr">
-        <is>
-          <t>Fortuna unnamed remaining 2025 (excl. seals $13,000 sold + Venus $20,000 sold + Belt $45,000 sold)</t>
-        </is>
-      </c>
-      <c r="C135" s="139" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="136" ht="14.25" customHeight="1" s="137"/>
+      <c r="E135" s="185" t="n"/>
+      <c r="F135" s="185" t="n"/>
+      <c r="G135" s="185" t="n"/>
+      <c r="H135" s="185" t="n"/>
+      <c r="I135" s="208" t="inlineStr">
+        <is>
+          <t>Moved to sold lots. Erdal 10/9 $25,000 / Cost $20,000 / net $5,000. Object unnamed. 11/7 $6,000 still ASK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="14.25" customHeight="1" s="137">
+      <c r="A136" s="206" t="inlineStr">
+        <is>
+          <t>Fortuna unnamed remaining 2025 (excl. seals $13,000 sold + Venus $20,000 sold + Belt $45,000 sold + August joint $20,000 sold)</t>
+        </is>
+      </c>
+      <c r="C136" s="183" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="137" ht="14.25" customHeight="1" s="137"/>
     <row r="138" ht="14.25" customHeight="1" s="137"/>
     <row r="139" ht="14.25" customHeight="1" s="137"/>
@@ -32317,8 +32376,8 @@
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A82:I82"/>
     <mergeCell ref="A119:I119"/>
-    <mergeCell ref="A81:I81"/>
     <mergeCell ref="A122:I122"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
Lock mosaics Cost $90k to Jamal from personal BoA.
User: $90k owed to Jamal (thinks $50k + $40k) sent from BoA 9922; $15k profit.
Plutus $50k on Mercury plus $40k personal; 2/24 $90k EPGC→9922 is funding, not extra Cost.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
+++ b/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
@@ -30,7 +30,6 @@
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="169" formatCode="_([$CAD]\ * #,##0.00_);_([$CAD]\ * \(#,##0.00\);_([$CAD]\ * &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="37">
     <font>
@@ -702,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="239">
+  <cellXfs count="240">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1210,6 +1209,9 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1786,7 +1788,7 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="182" t="inlineStr">
         <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $39,055.06 = prior MATCHED nets $23,055.06 (Berk lots + seals $1,000 + mosaics $15,000) + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 stays UNALLOCATED (per-invoice Deal Classifier; proposed FEE, no matching Cost — not dumped). Other L5 $37,396.32 / Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $39,055.06 = prior MATCHED nets $23,055.06 (Berk lots + seals $1,000 + mosaics $15,000) + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Mosaics Cost $90,000 LOCKED (Jamal via Plutus $50k on Mercury + personal BoA $40k); profit $15,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 stays UNALLOCATED (per-invoice Deal Classifier; proposed FEE, no matching Cost — not dumped). Other L5 $37,396.32 / Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -9670,7 +9672,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="238" t="inlineStr">
         <is>
@@ -24221,7 +24222,7 @@
     <row r="75" ht="84" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $251,000. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE, no matching dealer Cost; Fortuna joints are NOT EOEB Cost) — not dumped onto Consultant or Art Sales. Other L5 $37,396.32 MIXED — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD — cash on Art Sales, not in I8. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $251,000. Mosaics Cost $90,000 to Jamal LOCKED (Plutus $50k on 8291 + personal BoA $40k); profit $15,000 already in I8. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE) — not dumped. Other L5 $37,396.32 MIXED — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -30373,7 +30374,7 @@
       </c>
       <c r="I73" s="105" t="n"/>
     </row>
-    <row r="74" ht="14.25" customHeight="1" s="137">
+    <row r="74" ht="72" customHeight="1" s="137">
       <c r="A74" s="113" t="inlineStr">
         <is>
           <t>Three Ancient Mosaics</t>
@@ -30405,7 +30406,11 @@
         <f>SUM(F74-C74)</f>
         <v/>
       </c>
-      <c r="I74" s="105" t="n"/>
+      <c r="I74" s="239" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 Cost $90,000 to Jamal Rifai / DBA Antiquarium. User: the $90k owed to Jamal had to be sent from personal BoA 9922 (thinks $50k + $40k). Profit $15,000 ($105,000 EOEB 2/21 − $90,000 Cost). Payment: Mercury 8291 → Plutus &amp; Mnemosyne (DBA Antiquarium) 2/24–25 $50,000 + personal BoA $40,000. Mercury 2/24 $90,000 EPGC→9922 is same-day funding of personal — do NOT add as a second $90k of Cost. $40,000 of that transfer is mosaics Cost funding (not owner draw); $50,000 remains owner draw. Monarch 9922 has no labeled $40k outgoing to Jamal in Feb (only the $90k IN from EPGC) — confirm on 9922 stmt if needed. ASK 10 CLOSED. I8 already has mosaics net $15,000. Not tax advice.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="137">
       <c r="A75" s="113" t="inlineStr">
@@ -30648,7 +30653,7 @@
     <row r="82" ht="72" customHeight="1" s="137">
       <c r="A82" s="208" t="inlineStr">
         <is>
-          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics). Fortuna $13,000 (1/8 seals Cost). Plutus $50,000 of mosaics $90,000 Cost — $40,000 of Cost not on 8291 (ASK). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 (see Deal Classifier per invoice) or other L5 $37,396.32. Not tax advice.</t>
+          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics) / Cost $90,000 to Jamal (Plutus $50,000 on 8291 + personal BoA $40,000) / profit $15,000. Fortuna $13,000 (1/8 seals Cost). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 (see Deal Classifier per invoice) or other L5 $37,396.32. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -31251,19 +31256,6 @@
       <c r="A119" s="0" t="inlineStr">
         <is>
           <t>Hindman LLC (inventory purchase)</t>
-        </is>
-      </c>
-      <c r="B119" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C119" s="157" t="n">
-        <v>282.24</v>
-      </c>
-      <c r="D119" s="0" t="inlineStr">
-        <is>
-          <t>2025-04-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unbundle Plutus/Antiquarium as a second mosaic deal from Jamal.
EOEB 2/21 $105k stays pooled February Art Sales. Plutus $50k on Mercury is Deal B Cost, not a 40/50 Jamal mix. Combined $15k profit stays working; BoA 9922 draws restored to $261,172.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
+++ b/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
@@ -701,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="240">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1212,6 +1212,21 @@
     <xf numFmtId="9" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1788,7 +1803,7 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="182" t="inlineStr">
         <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $39,055.06 = prior MATCHED nets $23,055.06 (Berk lots + seals $1,000 + mosaics $15,000) + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Mosaics Cost $90,000 LOCKED (Jamal via Plutus $50k on Mercury + personal BoA $40k); profit $15,000. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 stays UNALLOCATED (per-invoice Deal Classifier; proposed FEE, no matching Cost — not dumped). Other L5 $37,396.32 / Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $39,055.06 = Berk lots + seals $1,000 + mosaics combined $15,000 WORKING + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Mosaics: TWO EOEB deals pooled in 2/21 $105,000. Plutus/Antiquarium $50k is Deal B Cost (not Jamal). Jamal Deal A Cost from personal BoA ASK. Combined profit $15k WORKING. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 stays UNALLOCATED (per-invoice Deal Classifier; proposed FEE, no matching Cost — not dumped). Other L5 $37,396.32 / Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -8662,7 +8677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="137" min="1" max="1"/>
@@ -9672,6 +9687,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="238" t="inlineStr">
         <is>
@@ -9825,6 +9841,13 @@
         </is>
       </c>
       <c r="D55" s="190" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mosaics 2026-09-21: TWO EOEB deals. Plutus/Antiquarium $50,000 on 8291 is Deal B Cost, not Jamal DBA. EOEB 2/21 $105,000 pooled SALE. Combined profit $15,000 WORKING in I8. Jamal BoA Cost amount ASK. 2/24 $90k EPGC→9922 is transfer, not extra Cost. Do not dump EOEB remainder $130,270. Not tax advice.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -24222,7 +24245,7 @@
     <row r="75" ht="84" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $251,000. Mosaics Cost $90,000 to Jamal LOCKED (Plutus $50k on 8291 + personal BoA $40k); profit $15,000 already in I8. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE) — not dumped. Other L5 $37,396.32 MIXED — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $251,000. Feb mosaics $105,000 is TWO EOEB deals pooled (Jamal + Plutus/Antiquarium). Plutus $50k on 8291 is Deal B Cost, not Jamal. Combined profit $15,000 WORKING in I8. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE) — not dumped. Other L5 $37,396.32 MIXED — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -30374,18 +30397,18 @@
       </c>
       <c r="I73" s="105" t="n"/>
     </row>
-    <row r="74" ht="72" customHeight="1" s="137">
-      <c r="A74" s="113" t="inlineStr">
-        <is>
-          <t>Three Ancient Mosaics</t>
-        </is>
-      </c>
-      <c r="B74" s="104" t="inlineStr">
-        <is>
-          <t>Jamal Rifai and Antiquarium</t>
-        </is>
-      </c>
-      <c r="C74" s="197" t="n">
+    <row r="74" ht="96" customHeight="1" s="137">
+      <c r="A74" s="240" t="inlineStr">
+        <is>
+          <t>Two mosaic deals (EOEB 2/21 pooled)</t>
+        </is>
+      </c>
+      <c r="B74" s="241" t="inlineStr">
+        <is>
+          <t>Jamal Rifai (Deal A) + Plutus/Antiquarium (Deal B)</t>
+        </is>
+      </c>
+      <c r="C74" s="242" t="n">
         <v>90000</v>
       </c>
       <c r="D74" s="115" t="n">
@@ -30396,7 +30419,7 @@
           <t>Jonathan Yantis</t>
         </is>
       </c>
-      <c r="F74" s="197" t="n">
+      <c r="F74" s="243" t="n">
         <v>105000</v>
       </c>
       <c r="G74" s="115" t="n">
@@ -30406,9 +30429,9 @@
         <f>SUM(F74-C74)</f>
         <v/>
       </c>
-      <c r="I74" s="239" t="inlineStr">
-        <is>
-          <t>LOCKED 2026-09-21 Cost $90,000 to Jamal Rifai / DBA Antiquarium. User: the $90k owed to Jamal had to be sent from personal BoA 9922 (thinks $50k + $40k). Profit $15,000 ($105,000 EOEB 2/21 − $90,000 Cost). Payment: Mercury 8291 → Plutus &amp; Mnemosyne (DBA Antiquarium) 2/24–25 $50,000 + personal BoA $40,000. Mercury 2/24 $90,000 EPGC→9922 is same-day funding of personal — do NOT add as a second $90k of Cost. $40,000 of that transfer is mosaics Cost funding (not owner draw); $50,000 remains owner draw. Monarch 9922 has no labeled $40k outgoing to Jamal in Feb (only the $90k IN from EPGC) — confirm on 9922 stmt if needed. ASK 10 CLOSED. I8 already has mosaics net $15,000. Not tax advice.</t>
+      <c r="I74" s="244" t="inlineStr">
+        <is>
+          <t>UNLOCKED 2026-09-21 40/50 mix. TWO mosaic deals, both EOEB. Deal A: Three Ancient Mosaics / Jamal Rifai — Cost paid from personal BoA (amount ASK). Deal B: Plutus &amp; Mnemosyne / DBA Antiquarium — Cost $50,000 on Mercury 8291 (2/24 $10 + 2/25 $49,990). EOEB 2/21 $105,000 MAKE A PAYMENT is pooled proceeds (user: perhaps paid for both at once). Do NOT treat Plutus as Jamal DBA. Combined Sale $105,000 LOCKED as February gross. Combined profit $15,000 WORKING (user; I8). Combined Cost $90,000 WORKING ($105k−$15k), not a locked Jamal 50+40. 2/24 $90k EPGC→9922 is owner transfer, not extra Cost. Monarch 9922 has no labeled $40k/$90k OUT to Jamal in Feb (only $90k IN from EPGC). Split of the $105k and Jamal BoA Cost still ASK. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -30650,10 +30673,10 @@
         <v/>
       </c>
     </row>
-    <row r="82" ht="72" customHeight="1" s="137">
-      <c r="A82" s="208" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB $105,000 (2/21 mosaics) / Cost $90,000 to Jamal (Plutus $50,000 on 8291 + personal BoA $40,000) / profit $15,000. Fortuna $13,000 (1/8 seals Cost). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 (see Deal Classifier per invoice) or other L5 $37,396.32. Not tax advice.</t>
+    <row r="82" ht="84" customHeight="1" s="137">
+      <c r="A82" s="190" t="inlineStr">
+        <is>
+          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB 2/21 $105,000 mosaics = TWO deals pooled (Jamal Deal A + Plutus/Antiquarium Deal B). Plutus $50,000 is Deal B Cost, not Jamal. Combined profit $15,000 WORKING in I8. Fortuna $13,000 (1/8 seals Cost). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 (see Deal Classifier per invoice) or other L5 $37,396.32. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock Q10 mosaics $50k/$40k/$15k and L5 leftovers as Consultant fees.
Recast the $15k mosaics slice out of Income I8 into EPGC Consultant February,
book L5 leftover invoices as fees, and leave remaining EOEB $108,270 unallocated.
Jamal Deal A Cost stays ASK. Belt, Venus, and August sales are unchanged.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
+++ b/.cursor/scratch/tax_turbo_deliverable/Personal Income 2025.xlsx
@@ -701,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="245">
+  <cellXfs count="246">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1227,6 +1227,9 @@
     <xf numFmtId="9" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1727,7 +1730,7 @@
         <v>20000</v>
       </c>
       <c r="I8" s="183" t="n">
-        <v>39055.06</v>
+        <v>24055.06</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="137">
@@ -1803,7 +1806,7 @@
     <row r="12" ht="48" customHeight="1" s="137">
       <c r="A12" s="182" t="inlineStr">
         <is>
-          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $39,055.06 = Berk lots + seals $1,000 + mosaics combined $15,000 WORKING + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Mosaics: TWO EOEB deals pooled in 2/21 $105,000. Plutus/Antiquarium $50k is Deal B Cost (not Jamal). Jamal Deal A Cost from personal BoA ASK. Combined profit $15k WORKING. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). EOEB remainder $130,270 stays UNALLOCATED (per-invoice Deal Classifier; proposed FEE, no matching Cost — not dumped). Other L5 $37,396.32 / Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $24,055.06 = Berk lots + seals $1,000 + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Mosaics $15,000 is FEE (EPGC Consultant February) — not I8. Deal B Plutus net $0. Deal A Jamal Cost ASK so not in I8. Excludes Sale 6428 $11,000 until Cost. Excludes Aquinas books $1,000 until Cost. David Aaron $13,595 is EPGC Consultant June (not I8). L5 leftover $37,396.32 / EOEB Canosan $1,000 / EOEB NBerk $21,000 are Consultant FEEs (not I8). EOEB remainder $108,270 stays UNALLOCATED (per-invoice Deal Classifier — not dumped). Erdal 11/7 $6,000 / Aysel $50,000 still ASK. Not tax advice.</t>
         </is>
       </c>
       <c r="B12" s="88" t="n"/>
@@ -8914,12 +8917,12 @@
       </c>
       <c r="C11" s="226" t="inlineStr">
         <is>
-          <t>39,055.06</t>
+          <t>24,055.06</t>
         </is>
       </c>
       <c r="D11" s="226" t="inlineStr">
         <is>
-          <t>Prior MATCHED $23,055.06 + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Sale 6428 and Aquinas wait on Cost.</t>
+          <t>Berk lots + seals $1,000 + Belt net $5,000 + Venus EPGC-share net $6,000 + August Fortuna joint net $5,000. Mosaics $15,000 is FEE (Consultant February), not I8. Deal A Cost ASK. Sale 6428 and Aquinas wait on Cost.</t>
         </is>
       </c>
       <c r="E11" s="226" t="inlineStr">
@@ -9265,12 +9268,12 @@
       </c>
       <c r="C24" s="226" t="inlineStr">
         <is>
-          <t>14,000 Jan + 136,000 Feb + 76,000 July + 25,000 Oct = 251,000</t>
+          <t>14,000 Jan + 121,000 Feb + 76,000 July + 25,000 Oct = 236,000</t>
         </is>
       </c>
       <c r="D24" s="226" t="inlineStr">
         <is>
-          <t>Gross sale cash. July = Belt L5 $50,000 + Venus $26,000. October = August Fortuna joint remittance $25,000. Do not dump EOEB $130,270 or other L5 $37,396.32.</t>
+          <t>Gross sale cash. Feb = Berk $30,000 + Aquinas $1,000 + mosaics SALE $90,000 (not the $15k FEE). July = Belt L5 $50,000 + Venus $26,000. October = August Fortuna joint remittance $25,000. Do not dump EOEB $108,270.</t>
         </is>
       </c>
       <c r="E24" s="226" t="inlineStr">
@@ -9287,17 +9290,17 @@
       </c>
       <c r="B25" s="224" t="inlineStr">
         <is>
-          <t>Consultant June</t>
+          <t>Consultant year</t>
         </is>
       </c>
       <c r="C25" s="224" t="inlineStr">
         <is>
-          <t>13,595.00</t>
+          <t>87,991.32</t>
         </is>
       </c>
       <c r="D25" s="224" t="inlineStr">
         <is>
-          <t>David Aaron Limited 6/24. User: consultant fee, not a sale.</t>
+          <t>Jan $1,000 Canosan + Feb $15,000 mosaics fee + May $21,000 NBerk + June $13,595 David Aaron + July $11,034.79 L5 + Sep $14,161.27 L5 + Oct $7,500 L5 + Dec $4,700.26 L5. Never I8.</t>
         </is>
       </c>
       <c r="E25" s="226" t="inlineStr">
@@ -9477,12 +9480,12 @@
     <row r="34">
       <c r="A34" s="224" t="inlineStr">
         <is>
-          <t>Dump EOEB $130,270 or other L5 $37,396.32 onto P&amp;L</t>
+          <t>Dump EOEB $108,270 onto P&amp;L</t>
         </is>
       </c>
       <c r="B34" s="224" t="inlineStr">
         <is>
-          <t>EOEB remainder is per-invoice UNALLOCATED (proposed FEE, no matching Cost). Not dumped. Belt $50k SALE; remaining L5 not attached.</t>
+          <t>EOEB remainder is per-invoice UNALLOCATED (proposed FEE, no matching Cost). Not dumped. Named FEEs are locked (Canosan $1k, NBerk $21k, mosaics $15k, L5 leftover $37,396.32). Belt $50k SALE; remaining L5 is FEE not attached to the belt.</t>
         </is>
       </c>
       <c r="C34" s="224" t="inlineStr"/>
@@ -9646,7 +9649,7 @@
         <v/>
       </c>
       <c r="C43" s="230" t="n">
-        <v>251000</v>
+        <v>236000</v>
       </c>
       <c r="D43" s="229">
         <f>IF(ROUND(B43,2)=ROUND(C43,2),"MATCH","FAIL")</f>
@@ -9665,7 +9668,7 @@
         <v/>
       </c>
       <c r="C44" s="230" t="n">
-        <v>13595</v>
+        <v>87991.32000000001</v>
       </c>
       <c r="D44" s="229">
         <f>IF(ROUND(B44,2)=ROUND(C44,2),"MATCH","FAIL")</f>
@@ -9687,7 +9690,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="238" t="inlineStr">
         <is>
@@ -9736,7 +9738,7 @@
       </c>
       <c r="D50" s="208" t="inlineStr">
         <is>
-          <t>Remaining L5 $37,396.32</t>
+          <t>Jamal Deal A Cost ASK</t>
         </is>
       </c>
     </row>
@@ -9775,12 +9777,12 @@
       </c>
       <c r="C52" s="208" t="inlineStr">
         <is>
-          <t>David Aaron June $13,595 Consultant; Wise write-ups $992.80 Fees</t>
+          <t>David Aaron June $13,595; mosaics $15,000 Feb; Canosan $1,000 Jan; NBerk $21,000 May; L5 leftover $37,396.32; Wise write-ups $992.80 Fees</t>
         </is>
       </c>
       <c r="D52" s="208" t="inlineStr">
         <is>
-          <t>EOEB remainder proposed FEE but not locked</t>
+          <t>EOEB remainder $108,270 proposed FEE but not locked</t>
         </is>
       </c>
     </row>
@@ -9815,12 +9817,12 @@
       </c>
       <c r="C54" s="190" t="inlineStr">
         <is>
-          <t>EOEB remainder $130,270.00 per-invoice (see DEAL_CLASSIFIER.csv)</t>
+          <t>EOEB remainder $108,270.00 per-invoice (see DEAL_CLASSIFIER.csv)</t>
         </is>
       </c>
       <c r="D54" s="190" t="inlineStr">
         <is>
-          <t>L5 remainder $37,396.32; Aysel $50,000</t>
+          <t>Erdal 11/7 $6,000; Aysel $50,000</t>
         </is>
       </c>
     </row>
@@ -9837,15 +9839,15 @@
       </c>
       <c r="C55" s="190" t="inlineStr">
         <is>
-          <t>EOEB remainder $130,270.00; other L5 $37,396.32; other Erdal IN $31,000; Aysel $50,000</t>
+          <t>EOEB remainder $108,270.00; Erdal 11/7 $6,000; Aysel $50,000</t>
         </is>
       </c>
       <c r="D55" s="190" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Mosaics 2026-09-21: TWO EOEB deals. Plutus/Antiquarium $50,000 on 8291 is Deal B Cost, not Jamal DBA. EOEB 2/21 $105,000 pooled SALE. Combined profit $15,000 WORKING in I8. Jamal BoA Cost amount ASK. 2/24 $90k EPGC→9922 is transfer, not extra Cost. Do not dump EOEB remainder $130,270. Not tax advice.</t>
+      <c r="A56" s="237" t="inlineStr">
+        <is>
+          <t>Mosaics 2026-09-21 LOCKED split: EOEB 2/21 $105,000 = Deal B Plutus/Antiquarium SALE $50,000 (Cost $50,000 on 8291, net $0) + Deal A Jamal SALE $40,000 (Cost ASK, not in I8) + $15,000 FEE (Consultant February, not I8 profit). Do not invent a $40k BoA Jamal Cost wire. 2/24 $90k EPGC→9922 is transfer, not extra Cost. Do not dump EOEB remainder $108,270. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -23428,8 +23430,8 @@
       <c r="B53" s="192" t="n">
         <v>14000</v>
       </c>
-      <c r="C53" s="192" t="n">
-        <v>136000</v>
+      <c r="C53" s="183" t="n">
+        <v>121000</v>
       </c>
       <c r="D53" s="179" t="n">
         <v>0</v>
@@ -23472,41 +23474,41 @@
           <t>Consultant</t>
         </is>
       </c>
-      <c r="B54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="C54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="192" t="n">
+      <c r="B54" s="183" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C54" s="183" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D54" s="192" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="192" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="183" t="n">
+        <v>21000</v>
+      </c>
+      <c r="G54" s="183" t="n">
         <v>13595</v>
       </c>
-      <c r="H54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="179" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="179" t="n">
-        <v>0</v>
+      <c r="H54" s="183" t="n">
+        <v>11034.79</v>
+      </c>
+      <c r="I54" s="192" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="183" t="n">
+        <v>14161.27</v>
+      </c>
+      <c r="K54" s="183" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L54" s="192" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="183" t="n">
+        <v>4700.26</v>
       </c>
       <c r="N54" s="193">
         <f>SUM(B54:M54)</f>
@@ -24245,7 +24247,7 @@
     <row r="75" ht="84" customHeight="1" s="137">
       <c r="A75" s="182" t="inlineStr">
         <is>
-          <t>2025 Mercury 2026-09-21: Art Sales gross cash by month = Jan $14,000 + Feb $136,000 MATCHED + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $251,000. Feb mosaics $105,000 is TWO EOEB deals pooled (Jamal + Plutus/Antiquarium). Plutus $50k on 8291 is Deal B Cost, not Jamal. Combined profit $15,000 WORKING in I8. Consultant June $13,595 = David Aaron Limited LOCKED (not a sale). Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $130,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE) — not dumped. Other L5 $37,396.32 MIXED — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
+          <t>2025 Mercury 2026-09-21 FEE lock: Art Sales gross cash by month = Jan $14,000 + Feb $121,000 (Berk $30,000 + Aquinas $1,000 + mosaics SALE $90,000) + July $76,000 (Belt L5 $50,000 + Venus remittance $26,000) + October $25,000 (August Fortuna joint remittance) = $236,000. EOEB 2/21 $105,000 split: Deal B $50,000 SALE + Deal A $40,000 SALE + $15,000 FEE. Consultant $87,991.32 = Jan $1,000 Canosan + Feb $15,000 mosaics fee + May $21,000 NBerk + June $13,595 David Aaron + July $11,034.79 L5 + Sep $14,161.27 L5 + Oct $7,500 L5 + Dec $4,700.26 L5. Consultant never to I8. Consultant Fees July $334.17 + October $658.63 = Wise expertise write-ups LOCKED ($992.80). EOEB remainder $108,270 is per-invoice UNALLOCATED on the Deal Classifier (proposed FEE) — not dumped. Erdal 11/7 $6,000 FORTUNA PAYMENT still ASK. Aysel Monarch +$50k vs native Failed −$50k still ASK (not the belt). Koziol/Ariadne $150,000 LOCKED pass-through — not P&amp;L. Coinbase is Investments. Newstar $23,581 is Art Sales COGS. Dec Wise $565.75 reimbursed. Aquinas books Cost TBD. Joint Sale Price = EPGC proceeds, not full hammer. GCM 1099 is personal. Not tax advice.</t>
         </is>
       </c>
     </row>
@@ -27794,7 +27796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z136"/>
+  <dimension ref="A1:Z137"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="47.86" customWidth="1" style="137" min="1" max="1"/>
@@ -30400,184 +30402,188 @@
     <row r="74" ht="96" customHeight="1" s="137">
       <c r="A74" s="240" t="inlineStr">
         <is>
-          <t>Two mosaic deals (EOEB 2/21 pooled)</t>
+          <t>Mosaic Deal B — Plutus/Antiquarium</t>
         </is>
       </c>
       <c r="B74" s="241" t="inlineStr">
         <is>
-          <t>Jamal Rifai (Deal A) + Plutus/Antiquarium (Deal B)</t>
-        </is>
-      </c>
-      <c r="C74" s="242" t="n">
-        <v>90000</v>
-      </c>
-      <c r="D74" s="115" t="n">
+          <t>Plutus &amp; Mnemosyne / DBA Antiquarium</t>
+        </is>
+      </c>
+      <c r="C74" s="243" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D74" s="245" t="n">
+        <v>45713</v>
+      </c>
+      <c r="E74" s="240" t="inlineStr">
+        <is>
+          <t>EOEB LLC</t>
+        </is>
+      </c>
+      <c r="F74" s="243" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G74" s="245" t="n">
         <v>45709</v>
       </c>
-      <c r="E74" s="113" t="inlineStr">
-        <is>
-          <t>Jonathan Yantis</t>
-        </is>
-      </c>
-      <c r="F74" s="243" t="n">
-        <v>105000</v>
-      </c>
-      <c r="G74" s="115" t="n">
+      <c r="H74" s="138">
+        <f>F74-C74</f>
+        <v/>
+      </c>
+      <c r="I74" s="244" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 SALE Deal B. Plutus &amp; Mnemosyne / DBA Antiquarium. Cost $50,000 on Mercury 8291 (2/24 $10 + 2/25 $49,990 native COGS). Sale $50,000 inside EOEB 2/21 $105,000 MAKE A PAYMENT (pooled with Deal A $40,000 SALE + $15,000 FEE). Net $0. Do NOT treat as Jamal DBA. 2/24 $90k EPGC→9922 is owner transfer, not extra Cost. Classifier: SALE. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="K74" s="178" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="96" customHeight="1" s="137">
+      <c r="A75" s="240" t="inlineStr">
+        <is>
+          <t>Mosaic Deal A — Three Ancient Mosaics / Jamal Rifai</t>
+        </is>
+      </c>
+      <c r="B75" s="241" t="inlineStr">
+        <is>
+          <t>Jamal M. Rifai (Cost ASK — personal BoA)</t>
+        </is>
+      </c>
+      <c r="C75" s="242" t="n"/>
+      <c r="D75" s="115" t="n"/>
+      <c r="E75" s="240" t="inlineStr">
+        <is>
+          <t>EOEB LLC</t>
+        </is>
+      </c>
+      <c r="F75" s="243" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G75" s="245" t="n">
         <v>45709</v>
       </c>
-      <c r="H74" s="88">
-        <f>SUM(F74-C74)</f>
-        <v/>
-      </c>
-      <c r="I74" s="244" t="inlineStr">
-        <is>
-          <t>UNLOCKED 2026-09-21 40/50 mix. TWO mosaic deals, both EOEB. Deal A: Three Ancient Mosaics / Jamal Rifai — Cost paid from personal BoA (amount ASK). Deal B: Plutus &amp; Mnemosyne / DBA Antiquarium — Cost $50,000 on Mercury 8291 (2/24 $10 + 2/25 $49,990). EOEB 2/21 $105,000 MAKE A PAYMENT is pooled proceeds (user: perhaps paid for both at once). Do NOT treat Plutus as Jamal DBA. Combined Sale $105,000 LOCKED as February gross. Combined profit $15,000 WORKING (user; I8). Combined Cost $90,000 WORKING ($105k−$15k), not a locked Jamal 50+40. 2/24 $90k EPGC→9922 is owner transfer, not extra Cost. Monarch 9922 has no labeled $40k/$90k OUT to Jamal in Feb (only $90k IN from EPGC). Split of the $105k and Jamal BoA Cost still ASK. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="14.25" customHeight="1" s="137">
-      <c r="A75" s="113" t="inlineStr">
-        <is>
-          <t>Canosan Terracotta Horse</t>
-        </is>
-      </c>
-      <c r="B75" s="104" t="inlineStr">
-        <is>
-          <t>Hindman</t>
-        </is>
-      </c>
-      <c r="C75" s="114" t="n">
-        <v>900</v>
-      </c>
-      <c r="D75" s="115" t="n"/>
-      <c r="E75" s="113" t="inlineStr">
-        <is>
-          <t>Erdal Dere</t>
-        </is>
-      </c>
-      <c r="F75" s="114" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G75" s="115" t="n"/>
-      <c r="H75" s="88">
-        <f>SUM(F75-C75)</f>
-        <v/>
-      </c>
-      <c r="I75" s="105" t="n"/>
+      <c r="H75" s="138">
+        <f>IF(OR(F75="",C75=""),"",F75-C75)</f>
+        <v/>
+      </c>
+      <c r="I75" s="244" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 SALE Deal A cash / ASK Cost. Three Ancient Mosaics / Jamal Rifai. Sale $40,000 inside EOEB 2/21 $105,000 (working dollars: $50k Antiquarium + $40k Jamal + $15k FEE). Cost from personal BoA still ASK — Monarch 9922 has no labeled $40k/$90k OUT to Jamal in Feb. Do not invent a $40k BoA Cost wire. $10 Mercury tests 2/21 and 2/24 only. Net excluded from I8 until Cost. The $15k is FEE (Consultant February), not art profit. Classifier: SALE. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="K75" s="178" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="137">
       <c r="A76" s="113" t="inlineStr">
         <is>
-          <t>Sale 6428 Contract 303468 (object TBD)</t>
+          <t>Canosan Terracotta Horse</t>
         </is>
       </c>
       <c r="B76" s="104" t="inlineStr">
         <is>
-          <t>Cost TBD</t>
-        </is>
-      </c>
-      <c r="C76" s="154" t="n"/>
+          <t>Hindman</t>
+        </is>
+      </c>
+      <c r="C76" s="114" t="n">
+        <v>900</v>
+      </c>
       <c r="D76" s="115" t="n"/>
       <c r="E76" s="113" t="inlineStr">
         <is>
+          <t>Erdal Dere</t>
+        </is>
+      </c>
+      <c r="F76" s="114" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G76" s="115" t="n"/>
+      <c r="H76" s="138">
+        <f>SUM(F76-C76)</f>
+        <v/>
+      </c>
+      <c r="I76" s="244" t="inlineStr">
+        <is>
+          <t>Register horse is Hindman Cost $900 sold to Erdal $1,000 (OPEN vs Berk 2/7 lump). EOEB 1/16 $1,000 is a FEE on Mercury 8291 — not this horse SALE. Do not double-count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="14.25" customHeight="1" s="137">
+      <c r="A77" s="113" t="inlineStr">
+        <is>
+          <t>Sale 6428 Contract 303468 (object TBD)</t>
+        </is>
+      </c>
+      <c r="B77" s="104" t="inlineStr">
+        <is>
+          <t>Cost TBD</t>
+        </is>
+      </c>
+      <c r="C77" s="154" t="n"/>
+      <c r="D77" s="115" t="n"/>
+      <c r="E77" s="113" t="inlineStr">
+        <is>
           <t>Freeman's LLC — check to Megan (joint 0203)</t>
         </is>
       </c>
-      <c r="F76" s="155" t="n">
+      <c r="F77" s="155" t="n">
         <v>11000</v>
       </c>
-      <c r="G76" s="115" t="inlineStr">
+      <c r="G77" s="115" t="inlineStr">
         <is>
           <t>2025-12-24</t>
         </is>
       </c>
-      <c r="H76" s="88">
-        <f>IF(C76="","",F76-C76)</f>
-        <v/>
-      </c>
-      <c r="I76" s="105" t="n"/>
-    </row>
-    <row r="77" ht="14.25" customHeight="1" s="137">
-      <c r="A77" s="181" t="inlineStr">
-        <is>
-          <t>Books (titles TBD)</t>
-        </is>
-      </c>
-      <c r="B77" s="185" t="inlineStr">
-        <is>
-          <t>Cost TBD</t>
-        </is>
-      </c>
-      <c r="C77" s="200" t="n"/>
-      <c r="E77" s="181" t="inlineStr">
-        <is>
-          <t>Aquinas Hobor</t>
-        </is>
-      </c>
-      <c r="F77" s="183" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G77" s="209" t="n">
-        <v>45692</v>
-      </c>
-      <c r="H77" s="178">
-        <f>IF(OR(F77="",C77=""),"",F77-C77)</f>
-        <v/>
-      </c>
-      <c r="I77" s="190" t="inlineStr">
-        <is>
-          <t>LOCKED 2026-09-20: book SALE $1,000 on Mercury 8291. Cost TBD — not in Income I8 yet (same as Sale 6428). Titles TBD. Not tax advice.</t>
-        </is>
-      </c>
+      <c r="H77" s="138">
+        <f>IF(C77="","",F77-C77)</f>
+        <v/>
+      </c>
+      <c r="I77" s="105" t="n"/>
     </row>
     <row r="78" ht="48" customHeight="1" s="137">
       <c r="A78" s="181" t="inlineStr">
         <is>
-          <t>Roman Gold Belt</t>
-        </is>
-      </c>
-      <c r="B78" s="181" t="inlineStr">
-        <is>
-          <t>Fortuna / Erdal Dere</t>
-        </is>
-      </c>
-      <c r="C78" s="183" t="n">
-        <v>45000</v>
-      </c>
-      <c r="D78" s="209" t="n">
-        <v>45859</v>
-      </c>
+          <t>Books (titles TBD)</t>
+        </is>
+      </c>
+      <c r="B78" s="185" t="inlineStr">
+        <is>
+          <t>Cost TBD</t>
+        </is>
+      </c>
+      <c r="C78" s="200" t="n"/>
       <c r="E78" s="181" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>Aquinas Hobor</t>
         </is>
       </c>
       <c r="F78" s="183" t="n">
-        <v>50000</v>
+        <v>1000</v>
       </c>
       <c r="G78" s="209" t="n">
-        <v>45853</v>
-      </c>
-      <c r="H78" s="183">
-        <f>F78-C78</f>
-        <v/>
-      </c>
-      <c r="I78" s="208" t="inlineStr">
-        <is>
-          <t>LOCKED 2026-09-21 SALE. Bought Fortuna/Erdal Dere 7/21 −$45,000 (Mercury 8291 native memo: Roman Gold Belt). Sold to L5. Working sale: L5 7/15 +$50,000 (only L5 payment large enough; L5 paid 6 days before Fortuna Cost — back-to-back dealer cash). Net $5,000. Do NOT attach remaining L5 invoices. Classifier: SALE. Not unsold inventory. Not consultant. Not pass-through. Not tax advice.</t>
-        </is>
-      </c>
-      <c r="J78" s="181" t="n"/>
-      <c r="K78" s="181" t="inlineStr">
-        <is>
-          <t>SALE</t>
+        <v>45692</v>
+      </c>
+      <c r="H78" s="138">
+        <f>IF(OR(F78="",C78=""),"",F78-C78)</f>
+        <v/>
+      </c>
+      <c r="I78" s="190" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-20: book SALE $1,000 on Mercury 8291. Cost TBD — not in Income I8 yet (same as Sale 6428). Titles TBD. Not tax advice.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1" s="137">
       <c r="A79" s="181" t="inlineStr">
         <is>
-          <t>Bronze head of a goddess, likely Venus (joint; EPGC share)</t>
+          <t>Roman Gold Belt</t>
         </is>
       </c>
       <c r="B79" s="181" t="inlineStr">
@@ -30586,21 +30592,21 @@
         </is>
       </c>
       <c r="C79" s="183" t="n">
-        <v>20000</v>
+        <v>45000</v>
       </c>
       <c r="D79" s="209" t="n">
-        <v>45786</v>
+        <v>45859</v>
       </c>
       <c r="E79" s="181" t="inlineStr">
         <is>
-          <t>Erdal Dere</t>
+          <t>L5</t>
         </is>
       </c>
       <c r="F79" s="183" t="n">
-        <v>26000</v>
+        <v>50000</v>
       </c>
       <c r="G79" s="209" t="n">
-        <v>45862</v>
+        <v>45853</v>
       </c>
       <c r="H79" s="183">
         <f>F79-C79</f>
@@ -30608,20 +30614,20 @@
       </c>
       <c r="I79" s="208" t="inlineStr">
         <is>
-          <t>LOCKED 2026-09-21 joint SALE (EPGC share). Erdal and Jacob bought together. EPGC Cost: Fortuna 5/9 −$20,000 (native memo: bronze head of a goddess, likely Venus). Erdal sold it and paid back Jacob’s investment plus earnings. Working remittance: Erdal Dere IN 7/24 +$26,000 = $20,000 investment + $6,000 earnings. Sale Price on this register is EPGC proceeds ($26,000), not the object’s full hammer. Classifier: SALE (joint, EPGC share). Not unsold inventory. Not consultant. Not tax advice.</t>
+          <t>LOCKED 2026-09-21 SALE. Bought Fortuna/Erdal Dere 7/21 −$45,000 (Mercury 8291 native memo: Roman Gold Belt). Sold to L5. Working sale: L5 7/15 +$50,000 (only L5 payment large enough; L5 paid 6 days before Fortuna Cost — back-to-back dealer cash). Net $5,000. Do NOT attach remaining L5 invoices. Classifier: SALE. Not unsold inventory. Not consultant. Not pass-through. Not tax advice.</t>
         </is>
       </c>
       <c r="J79" s="181" t="n"/>
       <c r="K79" s="181" t="inlineStr">
         <is>
-          <t>SALE (joint, EPGC share)</t>
+          <t>SALE</t>
         </is>
       </c>
     </row>
     <row r="80" ht="64" customHeight="1" s="137">
       <c r="A80" s="181" t="inlineStr">
         <is>
-          <t>August Fortuna joint — unnamed object (EPGC share)</t>
+          <t>Bronze head of a goddess, likely Venus (joint; EPGC share)</t>
         </is>
       </c>
       <c r="B80" s="181" t="inlineStr">
@@ -30633,7 +30639,7 @@
         <v>20000</v>
       </c>
       <c r="D80" s="209" t="n">
-        <v>45884</v>
+        <v>45786</v>
       </c>
       <c r="E80" s="181" t="inlineStr">
         <is>
@@ -30641,10 +30647,10 @@
         </is>
       </c>
       <c r="F80" s="183" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="G80" s="209" t="n">
-        <v>45939</v>
+        <v>45862</v>
       </c>
       <c r="H80" s="183">
         <f>F80-C80</f>
@@ -30652,7 +30658,7 @@
       </c>
       <c r="I80" s="208" t="inlineStr">
         <is>
-          <t>LOCKED 2026-09-21 joint SALE (EPGC share). Another joint investment with Erdal (user 2026-09-21). He sold; Jacob got capital + earnings. EPGC Cost: Fortuna 8/15 −$20,000 (Mercury native 8/18, same cash; object unnamed). Working remittance: Erdal Dere IN 10/9 +$25,000 = $20,000 capital + $5,000 earnings. Sale Price on this register is EPGC proceeds ($25,000), not the object’s full hammer. Hits EPGC Art Sales October. 7/24 is Venus, not August. 11/7 $6,000 FORTUNA PAYMENT still ASK. Classifier: SALE (joint, EPGC share). Not consultant. Not unsold inventory. Not tax advice.</t>
+          <t>LOCKED 2026-09-21 joint SALE (EPGC share). Erdal and Jacob bought together. EPGC Cost: Fortuna 5/9 −$20,000 (native memo: bronze head of a goddess, likely Venus). Erdal sold it and paid back Jacob’s investment plus earnings. Working remittance: Erdal Dere IN 7/24 +$26,000 = $20,000 investment + $6,000 earnings. Sale Price on this register is EPGC proceeds ($26,000), not the object’s full hammer. Classifier: SALE (joint, EPGC share). Not unsold inventory. Not consultant. Not tax advice.</t>
         </is>
       </c>
       <c r="J80" s="181" t="n"/>
@@ -30663,87 +30669,112 @@
       </c>
     </row>
     <row r="81" ht="64" customHeight="1" s="137">
-      <c r="A81" s="184" t="inlineStr">
+      <c r="A81" s="181" t="inlineStr">
+        <is>
+          <t>August Fortuna joint — unnamed object (EPGC share)</t>
+        </is>
+      </c>
+      <c r="B81" s="181" t="inlineStr">
+        <is>
+          <t>Fortuna / Erdal Dere</t>
+        </is>
+      </c>
+      <c r="C81" s="183" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D81" s="209" t="n">
+        <v>45884</v>
+      </c>
+      <c r="E81" s="181" t="inlineStr">
+        <is>
+          <t>Erdal Dere</t>
+        </is>
+      </c>
+      <c r="F81" s="183" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G81" s="209" t="n">
+        <v>45939</v>
+      </c>
+      <c r="H81" s="183">
+        <f>F81-C81</f>
+        <v/>
+      </c>
+      <c r="I81" s="208" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-09-21 joint SALE (EPGC share). Another joint investment with Erdal (user 2026-09-21). He sold; Jacob got capital + earnings. EPGC Cost: Fortuna 8/15 −$20,000 (Mercury native 8/18, same cash; object unnamed). Working remittance: Erdal Dere IN 10/9 +$25,000 = $20,000 capital + $5,000 earnings. Sale Price on this register is EPGC proceeds ($25,000), not the object’s full hammer. Hits EPGC Art Sales October. 7/24 is Venus, not August. 11/7 $6,000 FORTUNA PAYMENT still ASK. Classifier: SALE (joint, EPGC share). Not consultant. Not unsold inventory. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="J81" s="181" t="n"/>
+      <c r="K81" s="181" t="inlineStr">
+        <is>
+          <t>SALE (joint, EPGC share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="84" customHeight="1" s="137">
+      <c r="A82" s="184" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H81" s="235">
-        <f>SUM(H51:H75)+H78+H79+H80</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" ht="84" customHeight="1" s="137">
-      <c r="A82" s="190" t="inlineStr">
-        <is>
-          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB 2/21 $105,000 mosaics = TWO deals pooled (Jamal Deal A + Plutus/Antiquarium Deal B). Plutus $50,000 is Deal B Cost, not Jamal. Combined profit $15,000 WORKING in I8. Fortuna $13,000 (1/8 seals Cost). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant (EPGC Consultant June — not a sale). Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $130,270 (see Deal Classifier per invoice) or other L5 $37,396.32. Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="14.25" customHeight="1" s="137">
-      <c r="A83" s="119" t="inlineStr">
+      <c r="H82" s="138">
+        <f>SUM(H51:H76)+H79+H80+H81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" ht="96" customHeight="1" s="137">
+      <c r="A83" s="190" t="inlineStr">
+        <is>
+          <t>Mercury 8291 MATCHED/LOCKED: Berk $14,000 (1/10 seals) + $30,000 (2/7 lots). EOEB 2/21 $105,000 = Deal B Plutus SALE $50,000 + Deal A Jamal SALE $40,000 + $15,000 FEE (Consultant February — not I8). Plutus Cost $50,000 on 8291. Jamal Cost ASK (personal BoA). Fortuna $13,000 (1/8 seals Cost). Roman Gold Belt SALE to L5: Cost $45,000 / Sale $50,000 / net $5,000. Venus joint SALE EPGC share: Cost $20,000 / proceeds $26,000 / net $6,000. August Fortuna joint SALE EPGC share: Cost $20,000 / proceeds $25,000 / net $5,000 (Sale Price = remittance, not full hammer; object unnamed). L5 leftover $37,396.32 LOCKED FEE (Consultant; 7/15 $2,500 = 5% of belt; 10/21 $7,500 = 5% of Koziol/Ariadne). EOEB 1/16 $1,000 Canosan FEE (not horse SALE). EOEB 5/1 $21,000 NBerk FEE (not Venus). Newstar $23,581 jewelry fabrication COGS parked below. David Aaron $13,595 LOCKED consultant June. Aquinas Hobor $1,000 LOCKED book sale (Feb cash; Cost TBD, not in I8). Do not dump EOEB remainder $108,270 (see Deal Classifier per invoice). Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="14.25" customHeight="1" s="137">
+      <c r="A84" s="119" t="inlineStr">
         <is>
           <t>Art Purchases/Inventory</t>
         </is>
       </c>
-      <c r="B83" s="120" t="n"/>
-      <c r="C83" s="100" t="n"/>
-      <c r="D83" s="101" t="n"/>
-      <c r="E83" s="99" t="n"/>
-      <c r="F83" s="100" t="n"/>
-      <c r="G83" s="101" t="n"/>
-      <c r="H83" s="99" t="n"/>
-      <c r="I83" s="121" t="n"/>
-      <c r="J83" s="99" t="n"/>
-      <c r="K83" s="99" t="n"/>
-      <c r="L83" s="99" t="n"/>
-      <c r="M83" s="99" t="n"/>
-      <c r="N83" s="99" t="n"/>
-      <c r="O83" s="99" t="n"/>
-      <c r="P83" s="99" t="n"/>
-      <c r="Q83" s="99" t="n"/>
-      <c r="R83" s="99" t="n"/>
-      <c r="S83" s="99" t="n"/>
-      <c r="T83" s="99" t="n"/>
-      <c r="U83" s="99" t="n"/>
-      <c r="V83" s="99" t="n"/>
-      <c r="W83" s="99" t="n"/>
-      <c r="X83" s="99" t="n"/>
-      <c r="Y83" s="99" t="n"/>
-      <c r="Z83" s="99" t="n"/>
-    </row>
-    <row r="84" ht="14.25" customHeight="1" s="137">
-      <c r="A84" s="122" t="inlineStr">
-        <is>
-          <t>30 Paleothic and Neolithic Stone Tools</t>
-        </is>
-      </c>
-      <c r="B84" s="116" t="inlineStr">
-        <is>
-          <t>Holestein</t>
-        </is>
-      </c>
-      <c r="C84" s="88" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E84" s="105" t="n"/>
+      <c r="B84" s="120" t="n"/>
+      <c r="C84" s="100" t="n"/>
+      <c r="D84" s="101" t="n"/>
+      <c r="E84" s="99" t="n"/>
+      <c r="F84" s="100" t="n"/>
+      <c r="G84" s="101" t="n"/>
+      <c r="H84" s="99" t="n"/>
+      <c r="I84" s="121" t="n"/>
+      <c r="J84" s="99" t="n"/>
+      <c r="K84" s="99" t="n"/>
+      <c r="L84" s="99" t="n"/>
+      <c r="M84" s="99" t="n"/>
+      <c r="N84" s="99" t="n"/>
+      <c r="O84" s="99" t="n"/>
+      <c r="P84" s="99" t="n"/>
+      <c r="Q84" s="99" t="n"/>
+      <c r="R84" s="99" t="n"/>
+      <c r="S84" s="99" t="n"/>
+      <c r="T84" s="99" t="n"/>
+      <c r="U84" s="99" t="n"/>
+      <c r="V84" s="99" t="n"/>
+      <c r="W84" s="99" t="n"/>
+      <c r="X84" s="99" t="n"/>
+      <c r="Y84" s="99" t="n"/>
+      <c r="Z84" s="99" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1" s="137">
       <c r="A85" s="122" t="inlineStr">
         <is>
-          <t>A Tairona Figure</t>
+          <t>30 Paleothic and Neolithic Stone Tools</t>
         </is>
       </c>
       <c r="B85" s="116" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Holestein</t>
         </is>
       </c>
       <c r="C85" s="88" t="n">
-        <v>250</v>
-      </c>
-      <c r="D85" s="92" t="n">
-        <v>45119</v>
+        <v>4000</v>
       </c>
       <c r="E85" s="105" t="n"/>
     </row>
@@ -30759,7 +30790,7 @@
         </is>
       </c>
       <c r="C86" s="88" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D86" s="92" t="n">
         <v>45119</v>
@@ -30769,26 +30800,26 @@
     <row r="87" ht="14.25" customHeight="1" s="137">
       <c r="A87" s="122" t="inlineStr">
         <is>
-          <t>A Pair of Greek Bronze Greeves</t>
+          <t>A Tairona Figure</t>
         </is>
       </c>
       <c r="B87" s="116" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C87" s="88" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D87" s="92" t="n">
-        <v>45145</v>
+        <v>45119</v>
       </c>
       <c r="E87" s="105" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="137">
       <c r="A88" s="122" t="inlineStr">
         <is>
-          <t>An Illyrian Bronze Helmet</t>
+          <t>A Pair of Greek Bronze Greeves</t>
         </is>
       </c>
       <c r="B88" s="116" t="inlineStr">
@@ -30797,58 +30828,57 @@
         </is>
       </c>
       <c r="C88" s="88" t="n">
-        <v>551.25</v>
+        <v>200</v>
       </c>
       <c r="D88" s="92" t="n">
-        <v>45114</v>
+        <v>45145</v>
       </c>
       <c r="E88" s="105" t="n"/>
     </row>
     <row r="89" ht="14.25" customHeight="1" s="137">
       <c r="A89" s="122" t="inlineStr">
         <is>
-          <t>An Egyptian Faience Ibis</t>
-        </is>
-      </c>
-      <c r="B89" s="104" t="inlineStr">
-        <is>
-          <t>Hindman</t>
+          <t>An Illyrian Bronze Helmet</t>
+        </is>
+      </c>
+      <c r="B89" s="116" t="inlineStr">
+        <is>
+          <t>ebay</t>
         </is>
       </c>
       <c r="C89" s="88" t="n">
-        <v>375</v>
+        <v>551.25</v>
       </c>
       <c r="D89" s="92" t="n">
-        <v>44343</v>
-      </c>
-      <c r="E89" s="92" t="n"/>
-      <c r="F89" s="88" t="n"/>
-      <c r="I89" s="105" t="n"/>
+        <v>45114</v>
+      </c>
+      <c r="E89" s="105" t="n"/>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="137">
       <c r="A90" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
+          <t>An Egyptian Faience Ibis</t>
         </is>
       </c>
       <c r="B90" s="104" t="inlineStr">
         <is>
-          <t>Live Auctioneers</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C90" s="88" t="n">
-        <v>293</v>
+        <v>375</v>
       </c>
       <c r="D90" s="92" t="n">
-        <v>44548</v>
-      </c>
+        <v>44343</v>
+      </c>
+      <c r="E90" s="92" t="n"/>
       <c r="F90" s="88" t="n"/>
       <c r="I90" s="105" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="137">
       <c r="A91" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 1 0f 4</t>
         </is>
       </c>
       <c r="B91" s="104" t="inlineStr">
@@ -30868,7 +30898,7 @@
     <row r="92" ht="14.25" customHeight="1" s="137">
       <c r="A92" s="122" t="inlineStr">
         <is>
-          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
+          <t>African Stone Bracelet Upper Volta River 2 0f 4</t>
         </is>
       </c>
       <c r="B92" s="104" t="inlineStr">
@@ -30888,19 +30918,19 @@
     <row r="93" ht="14.25" customHeight="1" s="137">
       <c r="A93" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>African Stone Bracelet Upper Volta River 4 0f 4</t>
         </is>
       </c>
       <c r="B93" s="104" t="inlineStr">
         <is>
-          <t>Pace African Art</t>
+          <t>Live Auctioneers</t>
         </is>
       </c>
       <c r="C93" s="88" t="n">
-        <v>1000</v>
+        <v>293</v>
       </c>
       <c r="D93" s="92" t="n">
-        <v>44562</v>
+        <v>44548</v>
       </c>
       <c r="F93" s="88" t="n"/>
       <c r="I93" s="105" t="n"/>
@@ -30908,16 +30938,19 @@
     <row r="94" ht="14.25" customHeight="1" s="137">
       <c r="A94" s="122" t="inlineStr">
         <is>
-          <t>Carved Ostrish Egg</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B94" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etsy </t>
+          <t>Pace African Art</t>
         </is>
       </c>
       <c r="C94" s="88" t="n">
-        <v>90</v>
+        <v>1000</v>
+      </c>
+      <c r="D94" s="92" t="n">
+        <v>44562</v>
       </c>
       <c r="F94" s="88" t="n"/>
       <c r="I94" s="105" t="n"/>
@@ -30925,16 +30958,16 @@
     <row r="95" ht="14.25" customHeight="1" s="137">
       <c r="A95" s="122" t="inlineStr">
         <is>
-          <t>Carved Goose Egg</t>
+          <t>Carved Ostrish Egg</t>
         </is>
       </c>
       <c r="B95" s="104" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t xml:space="preserve">Etsy </t>
         </is>
       </c>
       <c r="C95" s="88" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="F95" s="88" t="n"/>
       <c r="I95" s="105" t="n"/>
@@ -30951,7 +30984,7 @@
         </is>
       </c>
       <c r="C96" s="88" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F96" s="88" t="n"/>
       <c r="I96" s="105" t="n"/>
@@ -30959,31 +30992,29 @@
     <row r="97" ht="14.25" customHeight="1" s="137">
       <c r="A97" s="122" t="inlineStr">
         <is>
-          <t>Quimbaya Figure (Gift)</t>
+          <t>Carved Goose Egg</t>
         </is>
       </c>
       <c r="B97" s="104" t="inlineStr">
         <is>
-          <t>Jeffrey Norris</t>
+          <t>Etsy</t>
         </is>
       </c>
       <c r="C97" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="D97" s="92" t="n">
-        <v>45079</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F97" s="88" t="n"/>
       <c r="I97" s="105" t="n"/>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="137">
       <c r="A98" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal (Gift)</t>
+          <t>Quimbaya Figure (Gift)</t>
         </is>
       </c>
       <c r="B98" s="104" t="inlineStr">
         <is>
-          <t>Aquinas Hobor</t>
+          <t>Jeffrey Norris</t>
         </is>
       </c>
       <c r="C98" s="88" t="n">
@@ -30997,7 +31028,7 @@
     <row r="99" ht="14.25" customHeight="1" s="137">
       <c r="A99" s="122" t="inlineStr">
         <is>
-          <t>A Saharan Stone Discoidal</t>
+          <t>A Saharan Stone Discoidal (Gift)</t>
         </is>
       </c>
       <c r="B99" s="104" t="inlineStr">
@@ -31005,31 +31036,30 @@
           <t>Aquinas Hobor</t>
         </is>
       </c>
-      <c r="C99" s="103" t="n">
-        <v>500</v>
+      <c r="C99" s="88" t="n">
+        <v>10</v>
       </c>
       <c r="D99" s="92" t="n">
         <v>45079</v>
       </c>
-      <c r="F99" s="88" t="n"/>
       <c r="I99" s="105" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1" s="137">
       <c r="A100" s="122" t="inlineStr">
         <is>
-          <t>Two Songye and Bozo Vessels</t>
+          <t>A Saharan Stone Discoidal</t>
         </is>
       </c>
       <c r="B100" s="104" t="inlineStr">
         <is>
-          <t>Hindman</t>
+          <t>Aquinas Hobor</t>
         </is>
       </c>
       <c r="C100" s="103" t="n">
-        <v>138.91</v>
+        <v>500</v>
       </c>
       <c r="D100" s="92" t="n">
-        <v>45211</v>
+        <v>45079</v>
       </c>
       <c r="F100" s="88" t="n"/>
       <c r="I100" s="105" t="n"/>
@@ -31037,19 +31067,19 @@
     <row r="101" ht="14.25" customHeight="1" s="137">
       <c r="A101" s="122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sword 9th Century </t>
+          <t>Two Songye and Bozo Vessels</t>
         </is>
       </c>
       <c r="B101" s="104" t="inlineStr">
         <is>
-          <t>Zevantiques</t>
+          <t>Hindman</t>
         </is>
       </c>
       <c r="C101" s="103" t="n">
-        <v>3000</v>
+        <v>138.91</v>
       </c>
       <c r="D101" s="92" t="n">
-        <v>45311</v>
+        <v>45211</v>
       </c>
       <c r="F101" s="88" t="n"/>
       <c r="I101" s="105" t="n"/>
@@ -31057,19 +31087,19 @@
     <row r="102" ht="14.25" customHeight="1" s="137">
       <c r="A102" s="122" t="inlineStr">
         <is>
-          <t>A Roman Marble Plaque with Insciption</t>
+          <t xml:space="preserve">Sword 9th Century </t>
         </is>
       </c>
       <c r="B102" s="104" t="inlineStr">
         <is>
-          <t>ebay</t>
+          <t>Zevantiques</t>
         </is>
       </c>
       <c r="C102" s="103" t="n">
-        <v>1331.41</v>
+        <v>3000</v>
       </c>
       <c r="D102" s="92" t="n">
-        <v>45546</v>
+        <v>45311</v>
       </c>
       <c r="F102" s="88" t="n"/>
       <c r="I102" s="105" t="n"/>
@@ -31077,7 +31107,7 @@
     <row r="103" ht="14.25" customHeight="1" s="137">
       <c r="A103" s="122" t="inlineStr">
         <is>
-          <t>Erotic Intaglio Finger Ring</t>
+          <t>A Roman Marble Plaque with Insciption</t>
         </is>
       </c>
       <c r="B103" s="104" t="inlineStr">
@@ -31086,85 +31116,94 @@
         </is>
       </c>
       <c r="C103" s="103" t="n">
-        <v>205.07</v>
+        <v>1331.41</v>
       </c>
       <c r="D103" s="92" t="n">
-        <v>45446</v>
+        <v>45546</v>
       </c>
       <c r="F103" s="88" t="n"/>
       <c r="I103" s="105" t="n"/>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="137">
-      <c r="B104" s="104" t="n"/>
-      <c r="C104" s="103" t="n"/>
-      <c r="D104" s="92" t="n"/>
+      <c r="A104" s="122" t="inlineStr">
+        <is>
+          <t>Erotic Intaglio Finger Ring</t>
+        </is>
+      </c>
+      <c r="B104" s="104" t="inlineStr">
+        <is>
+          <t>ebay</t>
+        </is>
+      </c>
+      <c r="C104" s="103" t="n">
+        <v>205.07</v>
+      </c>
+      <c r="D104" s="92" t="n">
+        <v>45446</v>
+      </c>
       <c r="F104" s="88" t="n"/>
       <c r="I104" s="105" t="n"/>
     </row>
     <row r="105" ht="14.25" customHeight="1" s="137">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
       <c r="B105" s="104" t="n"/>
-      <c r="C105" s="86" t="n"/>
+      <c r="C105" s="103" t="n"/>
+      <c r="D105" s="92" t="n"/>
       <c r="F105" s="88" t="n"/>
       <c r="I105" s="105" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="137">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
       <c r="B106" s="104" t="n"/>
-      <c r="C106" s="88" t="n"/>
+      <c r="C106" s="86" t="n"/>
       <c r="F106" s="88" t="n"/>
       <c r="I106" s="105" t="n"/>
     </row>
     <row r="107" ht="14.25" customHeight="1" s="137">
-      <c r="A107" s="119" t="inlineStr">
+      <c r="B107" s="104" t="n"/>
+      <c r="C107" s="88" t="n"/>
+      <c r="F107" s="88" t="n"/>
+      <c r="I107" s="105" t="n"/>
+    </row>
+    <row r="108" ht="14.25" customHeight="1" s="137">
+      <c r="A108" s="119" t="inlineStr">
         <is>
           <t>Office/Business Inventory</t>
         </is>
       </c>
-      <c r="B107" s="120" t="n"/>
-      <c r="C107" s="100" t="n"/>
-      <c r="D107" s="99" t="n"/>
-      <c r="E107" s="99" t="n"/>
-      <c r="F107" s="100" t="n"/>
-      <c r="G107" s="99" t="n"/>
-      <c r="H107" s="99" t="n"/>
-      <c r="I107" s="121" t="n"/>
-      <c r="J107" s="99" t="n"/>
-      <c r="K107" s="99" t="n"/>
-      <c r="L107" s="99" t="n"/>
-      <c r="M107" s="99" t="n"/>
-      <c r="N107" s="99" t="n"/>
-      <c r="O107" s="99" t="n"/>
-      <c r="P107" s="99" t="n"/>
-      <c r="Q107" s="99" t="n"/>
-      <c r="R107" s="99" t="n"/>
-      <c r="S107" s="99" t="n"/>
-      <c r="T107" s="99" t="n"/>
-      <c r="U107" s="99" t="n"/>
-      <c r="V107" s="99" t="n"/>
-      <c r="W107" s="99" t="n"/>
-      <c r="X107" s="99" t="n"/>
-      <c r="Y107" s="99" t="n"/>
-      <c r="Z107" s="99" t="n"/>
-    </row>
-    <row r="108" ht="14.25" customHeight="1" s="137">
-      <c r="A108" s="122" t="inlineStr">
-        <is>
-          <t>Sofa</t>
-        </is>
-      </c>
-      <c r="B108" s="104" t="n"/>
-      <c r="C108" s="88" t="n"/>
-      <c r="F108" s="88" t="n"/>
-      <c r="I108" s="105" t="n"/>
+      <c r="B108" s="120" t="n"/>
+      <c r="C108" s="100" t="n"/>
+      <c r="D108" s="99" t="n"/>
+      <c r="E108" s="99" t="n"/>
+      <c r="F108" s="100" t="n"/>
+      <c r="G108" s="99" t="n"/>
+      <c r="H108" s="99" t="n"/>
+      <c r="I108" s="121" t="n"/>
+      <c r="J108" s="99" t="n"/>
+      <c r="K108" s="99" t="n"/>
+      <c r="L108" s="99" t="n"/>
+      <c r="M108" s="99" t="n"/>
+      <c r="N108" s="99" t="n"/>
+      <c r="O108" s="99" t="n"/>
+      <c r="P108" s="99" t="n"/>
+      <c r="Q108" s="99" t="n"/>
+      <c r="R108" s="99" t="n"/>
+      <c r="S108" s="99" t="n"/>
+      <c r="T108" s="99" t="n"/>
+      <c r="U108" s="99" t="n"/>
+      <c r="V108" s="99" t="n"/>
+      <c r="W108" s="99" t="n"/>
+      <c r="X108" s="99" t="n"/>
+      <c r="Y108" s="99" t="n"/>
+      <c r="Z108" s="99" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1" s="137">
       <c r="A109" s="122" t="inlineStr">
         <is>
-          <t>Space Heater</t>
+          <t>Sofa</t>
         </is>
       </c>
       <c r="B109" s="104" t="n"/>
@@ -31175,7 +31214,7 @@
     <row r="110" ht="14.25" customHeight="1" s="137">
       <c r="A110" s="122" t="inlineStr">
         <is>
-          <t>Shelving</t>
+          <t>Space Heater</t>
         </is>
       </c>
       <c r="B110" s="104" t="n"/>
@@ -31186,7 +31225,7 @@
     <row r="111" ht="14.25" customHeight="1" s="137">
       <c r="A111" s="122" t="inlineStr">
         <is>
-          <t>Storage Bins</t>
+          <t>Shelving</t>
         </is>
       </c>
       <c r="B111" s="104" t="n"/>
@@ -31197,7 +31236,7 @@
     <row r="112" ht="14.25" customHeight="1" s="137">
       <c r="A112" s="122" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Storage Bins</t>
         </is>
       </c>
       <c r="B112" s="104" t="n"/>
@@ -31208,7 +31247,7 @@
     <row r="113" ht="14.25" customHeight="1" s="137">
       <c r="A113" s="122" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="B113" s="104" t="n"/>
@@ -31219,7 +31258,7 @@
     <row r="114" ht="14.25" customHeight="1" s="137">
       <c r="A114" s="122" t="inlineStr">
         <is>
-          <t>Art Library</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B114" s="104" t="n"/>
@@ -31230,7 +31269,7 @@
     <row r="115" ht="14.25" customHeight="1" s="137">
       <c r="A115" s="122" t="inlineStr">
         <is>
-          <t>Standing Desk</t>
+          <t>Art Library</t>
         </is>
       </c>
       <c r="B115" s="104" t="n"/>
@@ -31239,46 +31278,37 @@
       <c r="I115" s="105" t="n"/>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="137">
+      <c r="A116" s="122" t="inlineStr">
+        <is>
+          <t>Standing Desk</t>
+        </is>
+      </c>
       <c r="B116" s="104" t="n"/>
       <c r="C116" s="88" t="n"/>
       <c r="F116" s="88" t="n"/>
       <c r="I116" s="105" t="n"/>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="137">
-      <c r="A117" s="156" t="inlineStr">
-        <is>
-          <t>2025 CC inventory (not in Cost total until object is named)</t>
-        </is>
-      </c>
       <c r="B117" s="104" t="n"/>
       <c r="C117" s="88" t="n"/>
       <c r="F117" s="88" t="n"/>
       <c r="I117" s="105" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1" s="137">
-      <c r="A118" s="0" t="inlineStr">
-        <is>
-          <t>Los Angeles Modern Auctions (inventory purchase)</t>
-        </is>
-      </c>
-      <c r="B118" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C118" s="157" t="n">
-        <v>6821.06</v>
-      </c>
-      <c r="D118" s="0" t="inlineStr">
-        <is>
-          <t>2025-07-24</t>
-        </is>
-      </c>
+      <c r="A118" s="156" t="inlineStr">
+        <is>
+          <t>2025 CC inventory (not in Cost total until object is named)</t>
+        </is>
+      </c>
+      <c r="B118" s="104" t="n"/>
+      <c r="C118" s="88" t="n"/>
+      <c r="F118" s="88" t="n"/>
+      <c r="I118" s="105" t="n"/>
     </row>
     <row r="119" ht="14.25" customHeight="1" s="137">
       <c r="A119" s="0" t="inlineStr">
         <is>
-          <t>Hindman LLC (inventory purchase)</t>
+          <t>Los Angeles Modern Auctions (inventory purchase)</t>
         </is>
       </c>
     </row>
@@ -31292,84 +31322,53 @@
     <row r="121" ht="14.25" customHeight="1" s="137">
       <c r="A121" s="0" t="inlineStr">
         <is>
+          <t>Hindman LLC (inventory purchase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="14.25" customHeight="1" s="137">
+      <c r="A122" s="0" t="inlineStr">
+        <is>
           <t>The Great Frame Up (inventory framing)</t>
         </is>
       </c>
-      <c r="B121" s="0" t="inlineStr">
-        <is>
-          <t>Sapphire 5423</t>
-        </is>
-      </c>
-      <c r="C121" s="157" t="n">
-        <v>536.41</v>
-      </c>
-      <c r="D121" s="0" t="inlineStr">
-        <is>
-          <t>2025-02-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="14.25" customHeight="1" s="137"/>
-    <row r="123" ht="14.25" customHeight="1" s="137">
-      <c r="A123" s="201" t="inlineStr">
+    </row>
+    <row r="123" ht="14.25" customHeight="1" s="137"/>
+    <row r="124" ht="14.25" customHeight="1" s="137">
+      <c r="A124" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury 8291 — David Aaron Limited is LOCKED consultant fee (not Art Sales)</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="14.25" customHeight="1" s="137">
-      <c r="A124" s="181" t="inlineStr">
+    <row r="125" ht="14.25" customHeight="1" s="137">
+      <c r="A125" s="181" t="inlineStr">
         <is>
           <t>NOT a 2025 art sale — David Aaron Limited consultant fee (EPGC Consultant June)</t>
         </is>
       </c>
-      <c r="B124" s="181" t="inlineStr">
+      <c r="B125" s="181" t="inlineStr">
         <is>
           <t>David Aaron Limited</t>
         </is>
       </c>
-      <c r="C124" s="181" t="n"/>
-      <c r="D124" s="181" t="n"/>
-      <c r="E124" s="181" t="n"/>
-      <c r="F124" s="183" t="n"/>
-      <c r="G124" s="206" t="n"/>
-      <c r="H124" s="206" t="n"/>
-      <c r="I124" s="181" t="inlineStr">
+      <c r="C125" s="181" t="n"/>
+      <c r="D125" s="181" t="n"/>
+      <c r="E125" s="181" t="n"/>
+      <c r="F125" s="183" t="n"/>
+      <c r="G125" s="206" t="n"/>
+      <c r="H125" s="206" t="n"/>
+      <c r="I125" s="181" t="inlineStr">
         <is>
           <t>LOCKED 2026-09-20: consultant fee, not a sale. $13,595 is on EPGC Consultant June. Not tax advice.</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="14.25" customHeight="1" s="137"/>
-    <row r="126" ht="14.25" customHeight="1" s="137">
-      <c r="A126" s="201" t="inlineStr">
+    <row r="126" ht="14.25" customHeight="1" s="137"/>
+    <row r="127" ht="14.25" customHeight="1" s="137">
+      <c r="A127" s="201" t="inlineStr">
         <is>
           <t>2025 Mercury COGS — Newstar Jewelers (LOCKED jewelry fabrication)</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="14.25" customHeight="1" s="137">
-      <c r="A127" s="202" t="inlineStr">
-        <is>
-          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
-        </is>
-      </c>
-      <c r="B127" s="202" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C127" s="203" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D127" s="202" t="inlineStr">
-        <is>
-          <t>2025-10-14</t>
-        </is>
-      </c>
-      <c r="I127" s="0" t="inlineStr">
-        <is>
-          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
@@ -31389,7 +31388,7 @@
       </c>
       <c r="D128" s="202" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="I128" s="0" t="inlineStr">
@@ -31401,74 +31400,76 @@
     <row r="129" ht="14.25" customHeight="1" s="137">
       <c r="A129" s="202" t="inlineStr">
         <is>
+          <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs</t>
+        </is>
+      </c>
+      <c r="B129" s="202" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C129" s="203" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D129" s="202" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
+      <c r="I129" s="0" t="inlineStr">
+        <is>
+          <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="14.25" customHeight="1" s="137">
+      <c r="A130" s="202" t="inlineStr">
+        <is>
           <t>Newstar Jewelers — jewelry from intaglios / engraved gems / scarabs (3 of 3)</t>
         </is>
       </c>
-      <c r="B129" s="202" t="inlineStr">
+      <c r="B130" s="202" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C129" s="203" t="n">
+      <c r="C130" s="203" t="n">
         <v>7581</v>
       </c>
-      <c r="D129" s="202" t="inlineStr">
+      <c r="D130" s="202" t="inlineStr">
         <is>
           <t>2025-12-24</t>
         </is>
       </c>
-      <c r="I129" s="0" t="inlineStr">
+      <c r="I130" s="0" t="inlineStr">
         <is>
           <t>LOCKED COGS fabrication. Not in sold-lot Cost total (Feb Berk lots already sold). Identify which gems/intaglios/scarabs.</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="14.25" customHeight="1" s="137">
-      <c r="A130" s="0" t="inlineStr">
+    <row r="131" ht="14.25" customHeight="1" s="137">
+      <c r="A131" s="0" t="inlineStr">
         <is>
           <t>Newstar 2025 total</t>
         </is>
       </c>
-      <c r="C130" s="183">
+      <c r="C131" s="183">
         <f>SUM(C127:C129)</f>
         <v/>
       </c>
     </row>
-    <row r="131" ht="14.25" customHeight="1" s="137"/>
-    <row r="132" ht="14.25" customHeight="1" s="137">
-      <c r="A132" s="236" t="inlineStr">
+    <row r="132" ht="14.25" customHeight="1" s="137"/>
+    <row r="133" ht="14.25" customHeight="1" s="137">
+      <c r="A133" s="236" t="inlineStr">
         <is>
           <t>2025 Mercury Fortuna — Venus + Belt + August joint SOLD 2025 (see Sales 2025 rows 78–80); no unnamed Fortuna Cost left on 8291</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="14.25" customHeight="1" s="137">
-      <c r="A133" s="181" t="inlineStr">
-        <is>
-          <t>SOLD 2025 — Venus joint (see Sales 2025 row 79). Not unsold inventory.</t>
-        </is>
-      </c>
-      <c r="B133" s="181" t="inlineStr">
-        <is>
-          <t>Mercury 8291</t>
-        </is>
-      </c>
-      <c r="C133" s="183" t="n"/>
-      <c r="D133" s="202" t="inlineStr">
-        <is>
-          <t>2025-05-09</t>
-        </is>
-      </c>
-      <c r="I133" s="208" t="inlineStr">
-        <is>
-          <t>Moved to sold lots. EPGC proceeds $26,000 / Cost $20,000 / net $6,000.</t>
         </is>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="137">
       <c r="A134" s="181" t="inlineStr">
         <is>
-          <t>SOLD 2025 — Roman Gold Belt to L5 (see Sales 2025 row 78). Not unsold inventory.</t>
+          <t>SOLD 2025 — Venus joint (see Sales 2025 row 79). Not unsold inventory.</t>
         </is>
       </c>
       <c r="B134" s="181" t="inlineStr">
@@ -31479,53 +31480,75 @@
       <c r="C134" s="183" t="n"/>
       <c r="D134" s="202" t="inlineStr">
         <is>
-          <t>2025-07-21</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="I134" s="208" t="inlineStr">
         <is>
-          <t>Moved to sold lots. L5 $50,000 / Cost $45,000 / net $5,000. Remaining L5 not attached.</t>
+          <t>Moved to sold lots. EPGC proceeds $26,000 / Cost $20,000 / net $6,000.</t>
         </is>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="137">
       <c r="A135" s="181" t="inlineStr">
         <is>
+          <t>SOLD 2025 — Roman Gold Belt to L5 (see Sales 2025 row 78). Not unsold inventory.</t>
+        </is>
+      </c>
+      <c r="B135" s="181" t="inlineStr">
+        <is>
+          <t>Mercury 8291</t>
+        </is>
+      </c>
+      <c r="C135" s="183" t="n"/>
+      <c r="D135" s="202" t="inlineStr">
+        <is>
+          <t>2025-07-21</t>
+        </is>
+      </c>
+      <c r="I135" s="208" t="inlineStr">
+        <is>
+          <t>Moved to sold lots. L5 $50,000 / Cost $45,000 / net $5,000. Remaining L5 not attached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="14.25" customHeight="1" s="137">
+      <c r="A136" s="181" t="inlineStr">
+        <is>
           <t>SOLD 2025 — August Fortuna joint (see Sales 2025 row 80). Not unsold inventory.</t>
         </is>
       </c>
-      <c r="B135" s="185" t="inlineStr">
+      <c r="B136" s="185" t="inlineStr">
         <is>
           <t>Mercury 8291</t>
         </is>
       </c>
-      <c r="C135" s="183" t="n"/>
-      <c r="D135" s="185" t="inlineStr">
+      <c r="C136" s="183" t="n"/>
+      <c r="D136" s="185" t="inlineStr">
         <is>
           <t>2025-08-15</t>
         </is>
       </c>
-      <c r="E135" s="185" t="n"/>
-      <c r="F135" s="185" t="n"/>
-      <c r="G135" s="185" t="n"/>
-      <c r="H135" s="185" t="n"/>
-      <c r="I135" s="208" t="inlineStr">
+      <c r="E136" s="185" t="n"/>
+      <c r="F136" s="185" t="n"/>
+      <c r="G136" s="185" t="n"/>
+      <c r="H136" s="185" t="n"/>
+      <c r="I136" s="208" t="inlineStr">
         <is>
           <t>Moved to sold lots. Erdal 10/9 $25,000 / Cost $20,000 / net $5,000. Object unnamed. 11/7 $6,000 still ASK.</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="14.25" customHeight="1" s="137">
-      <c r="A136" s="206" t="inlineStr">
+    <row r="137" ht="14.25" customHeight="1" s="137">
+      <c r="A137" s="206" t="inlineStr">
         <is>
           <t>Fortuna unnamed remaining 2025 (excl. seals $13,000 sold + Venus $20,000 sold + Belt $45,000 sold + August joint $20,000 sold)</t>
         </is>
       </c>
-      <c r="C136" s="183" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" ht="14.25" customHeight="1" s="137"/>
+      <c r="C137" s="183" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="138" ht="14.25" customHeight="1" s="137"/>
     <row r="139" ht="14.25" customHeight="1" s="137"/>
     <row r="140" ht="14.25" customHeight="1" s="137"/>
@@ -32391,7 +32414,7 @@
     <row r="1000" ht="14.25" customHeight="1" s="137"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A82:I82"/>
+    <mergeCell ref="A83:I83"/>
     <mergeCell ref="A119:I119"/>
     <mergeCell ref="A122:I122"/>
   </mergeCells>

</xml_diff>